<commit_message>
Update TS Train and Test data files
</commit_message>
<xml_diff>
--- a/Early cancer detection/TS Test.xlsx
+++ b/Early cancer detection/TS Test.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30106"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\01_PhD\BaiduSyncdisk\PhD\09_文章数据\TS Prediction_RF_LDA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSoft\Pycharm\PythonProject\PythonProject\Archive\01_tri_cancer_screening\Source code for submission\Early cancer detection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F242825A-261E-415D-9246-17692E1D1C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BFEC10C-6828-4873-8F29-D44C191C1AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9132" yWindow="1344" windowWidth="19320" windowHeight="14616" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="15">
   <si>
     <t>LuC</t>
   </si>
@@ -78,196 +77,6 @@
     <t>dwl(6,4)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
-  <si>
-    <t>(6,4)-X23__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X24__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X11__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X13__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X14__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X15__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X16__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X17__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X18__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X20__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X21__660</t>
-  </si>
-  <si>
-    <t>(6,4)-X22__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N1__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N10__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N11__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N12__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N13__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N14__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N15__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N16__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N17__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N18__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N19__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N2__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N20__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N3__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N4__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N5__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N6__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N7__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N8__660</t>
-  </si>
-  <si>
-    <t>(6,4)-N9__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N1__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N10__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N11__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N12__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N13__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N14__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N15__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N16__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N17__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N18__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N19__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N2__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N20__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N21__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N22__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N23__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N24__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N25__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N26__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N27__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N28__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N29__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N3__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N30__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N4__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N5__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N6__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N7__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N8__660</t>
-  </si>
-  <si>
-    <t>(9,1)-N9__660</t>
-  </si>
-  <si>
-    <t>N</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
 </sst>
 </file>
 
@@ -276,7 +85,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -371,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -391,9 +200,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -406,12 +212,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -693,12 +493,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N78"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="14" max="14" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -739,499 +539,499 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="9">
         <v>-1.41622</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="9">
         <v>-1.35989</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="9">
         <v>0.49380000000000002</v>
       </c>
-      <c r="E2" s="10">
+      <c r="E2" s="9">
         <v>-1.5841099999999999</v>
       </c>
-      <c r="F2" s="10">
+      <c r="F2" s="9">
         <v>0.49720999999999999</v>
       </c>
-      <c r="G2" s="10">
+      <c r="G2" s="9">
         <v>0.57604</v>
       </c>
-      <c r="H2" s="11">
+      <c r="H2" s="10">
         <v>-0.40747</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="9">
         <v>-1.2265900000000001</v>
       </c>
-      <c r="J2" s="10">
+      <c r="J2" s="9">
         <v>8.1449999999999995E-2</v>
       </c>
-      <c r="K2" s="10">
+      <c r="K2" s="9">
         <v>3.9453100000000001</v>
       </c>
-      <c r="L2" s="10">
+      <c r="L2" s="9">
         <v>-0.29224</v>
       </c>
-      <c r="M2" s="10">
+      <c r="M2" s="9">
         <v>-5.0499999999999998E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="7">
         <v>0.30044999999999999</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="7">
         <v>1.7805500000000001</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="7">
         <v>0.65408999999999995</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="7">
         <v>-1.4532</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="7">
         <v>0.51732999999999996</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="7">
         <v>0.91549000000000003</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="8">
         <v>-1.4694</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="7">
         <v>-0.77751999999999999</v>
       </c>
-      <c r="J3" s="8">
+      <c r="J3" s="7">
         <v>0.19339000000000001</v>
       </c>
-      <c r="K3" s="8">
+      <c r="K3" s="7">
         <v>2.21698</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="7">
         <v>4.1980000000000003E-2</v>
       </c>
-      <c r="M3" s="8">
+      <c r="M3" s="7">
         <v>0.12911</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="7">
         <v>-0.33622999999999997</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <v>0.94950000000000001</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="7">
         <v>0.30614000000000002</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="7">
         <v>-1.4003000000000001</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="7">
         <v>0.28273999999999999</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <v>0.54825999999999997</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="8">
         <v>-1.6550199999999999</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="7">
         <v>-0.66008999999999995</v>
       </c>
-      <c r="J4" s="8">
+      <c r="J4" s="7">
         <v>0.22846</v>
       </c>
-      <c r="K4" s="8">
+      <c r="K4" s="7">
         <v>2.12697</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="7">
         <v>4.3770000000000003E-2</v>
       </c>
-      <c r="M4" s="8">
+      <c r="M4" s="7">
         <v>0.18670999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="7">
         <v>0.87195</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <v>1.7372399999999999</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="7">
         <v>0.62536000000000003</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="7">
         <v>-1.6284700000000001</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="7">
         <v>0.33001999999999998</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="7">
         <v>1.00159</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="8">
         <v>-1.2565500000000001</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="7">
         <v>-0.72762000000000004</v>
       </c>
-      <c r="J5" s="8">
+      <c r="J5" s="7">
         <v>0.33993000000000001</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5" s="7">
         <v>2.5489799999999998</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="7">
         <v>0.16298000000000001</v>
       </c>
-      <c r="M5" s="8">
+      <c r="M5" s="7">
         <v>0.28004000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="7">
         <v>6.4269999999999994E-2</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="7">
         <v>1.7006300000000001</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="7">
         <v>-5.6030000000000003E-2</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <v>-1.0752299999999999</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="7">
         <v>0.50238000000000005</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="7">
         <v>0.81172999999999995</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="8">
         <v>-1.6113200000000001</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="7">
         <v>-1.4603299999999999</v>
       </c>
-      <c r="J6" s="8">
+      <c r="J6" s="7">
         <v>0.14982999999999999</v>
       </c>
-      <c r="K6" s="8">
+      <c r="K6" s="7">
         <v>1.29216</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="7">
         <v>0.37297000000000002</v>
       </c>
-      <c r="M6" s="8">
+      <c r="M6" s="7">
         <v>0.12698000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="7">
         <v>-0.10381</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="7">
         <v>1.0991200000000001</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="7">
         <v>0.25996000000000002</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="7">
         <v>-1.4366399999999999</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="7">
         <v>0.26889000000000002</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="7">
         <v>0.73860000000000003</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="8">
         <v>-1.53294</v>
       </c>
-      <c r="I7" s="8">
+      <c r="I7" s="7">
         <v>-1.0687800000000001</v>
       </c>
-      <c r="J7" s="8">
+      <c r="J7" s="7">
         <v>0.20599999999999999</v>
       </c>
-      <c r="K7" s="8">
+      <c r="K7" s="7">
         <v>1.9022300000000001</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="7">
         <v>3.2960000000000003E-2</v>
       </c>
-      <c r="M7" s="8">
+      <c r="M7" s="7">
         <v>0.12474</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="7">
         <v>0.84330000000000005</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="7">
         <v>1.2326299999999999</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="7">
         <v>0.82532000000000005</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="7">
         <v>-1.5825800000000001</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="7">
         <v>0.36374000000000001</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="7">
         <v>1.01393</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H8" s="8">
         <v>-1.3601700000000001</v>
       </c>
-      <c r="I8" s="8">
+      <c r="I8" s="7">
         <v>-0.85970000000000002</v>
       </c>
-      <c r="J8" s="8">
+      <c r="J8" s="7">
         <v>0.23035</v>
       </c>
-      <c r="K8" s="8">
+      <c r="K8" s="7">
         <v>2.4791699999999999</v>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="7">
         <v>0.42114000000000001</v>
       </c>
-      <c r="M8" s="8">
+      <c r="M8" s="7">
         <v>0.20910999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="7">
         <v>-1.81494</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="7">
         <v>1.4992099999999999</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="7">
         <v>-1.1259399999999999</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="7">
         <v>-1.0402899999999999</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="7">
         <v>0.39118000000000003</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="7">
         <v>0.58652000000000004</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="8">
         <v>-1.6991499999999999</v>
       </c>
-      <c r="I9" s="8">
+      <c r="I9" s="7">
         <v>-1.4641500000000001</v>
       </c>
-      <c r="J9" s="8">
+      <c r="J9" s="7">
         <v>0.54198999999999997</v>
       </c>
-      <c r="K9" s="8">
+      <c r="K9" s="7">
         <v>1.0265200000000001</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="7">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="M9" s="8">
+      <c r="M9" s="7">
         <v>5.8090000000000003E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="7">
         <v>-2.0194000000000001</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="7">
         <v>1.0533999999999999</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="7">
         <v>-1.3171200000000001</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="7">
         <v>-1.3277000000000001</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="7">
         <v>0.15129000000000001</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="7">
         <v>0.25361</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="8">
         <v>-1.8179700000000001</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="7">
         <v>-0.63066999999999995</v>
       </c>
-      <c r="J10" s="8">
+      <c r="J10" s="7">
         <v>0.46848000000000001</v>
       </c>
-      <c r="K10" s="8">
+      <c r="K10" s="7">
         <v>1.49057</v>
       </c>
-      <c r="L10" s="8">
+      <c r="L10" s="7">
         <v>5.5070000000000001E-2</v>
       </c>
-      <c r="M10" s="8">
+      <c r="M10" s="7">
         <v>2.913E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="7">
         <v>-1.6923299999999999</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="7">
         <v>1.6949099999999999</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="7">
         <v>-0.52973000000000003</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="7">
         <v>-0.94506000000000001</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="7">
         <v>0.34649999999999997</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="7">
         <v>0.88263000000000003</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="8">
         <v>-1.5450999999999999</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="7">
         <v>-0.64778999999999998</v>
       </c>
-      <c r="J11" s="8">
+      <c r="J11" s="7">
         <v>0.51185999999999998</v>
       </c>
-      <c r="K11" s="8">
+      <c r="K11" s="7">
         <v>1.25708</v>
       </c>
-      <c r="L11" s="8">
+      <c r="L11" s="7">
         <v>0.22914000000000001</v>
       </c>
-      <c r="M11" s="8">
+      <c r="M11" s="7">
         <v>0.14810000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="7">
         <v>-1.43852</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="7">
         <v>2.0183399999999998</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="7">
         <v>-0.48720999999999998</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="7">
         <v>-0.52761999999999998</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="7">
         <v>0.45629999999999998</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="7">
         <v>0.80808999999999997</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="8">
         <v>-1.4275800000000001</v>
       </c>
-      <c r="I12" s="8">
+      <c r="I12" s="7">
         <v>-1.7190700000000001</v>
       </c>
-      <c r="J12" s="8">
+      <c r="J12" s="7">
         <v>0.61511000000000005</v>
       </c>
-      <c r="K12" s="8">
+      <c r="K12" s="7">
         <v>1.01118</v>
       </c>
-      <c r="L12" s="8">
+      <c r="L12" s="7">
         <v>9.5100000000000004E-2</v>
       </c>
-      <c r="M12" s="8">
+      <c r="M12" s="7">
         <v>-6.9339999999999999E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="7">
         <v>-1.87588</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="7">
         <v>1.15892</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="7">
         <v>-0.96457999999999999</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="7">
         <v>-1.02505</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="7">
         <v>0.18890000000000001</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="7">
         <v>0.47039999999999998</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="8">
         <v>-1.72149</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="7">
         <v>-0.90486999999999995</v>
       </c>
-      <c r="J13" s="8">
+      <c r="J13" s="7">
         <v>0.43490000000000001</v>
       </c>
-      <c r="K13" s="8">
+      <c r="K13" s="7">
         <v>1.09406</v>
       </c>
-      <c r="L13" s="8">
+      <c r="L13" s="7">
         <v>0.24060000000000001</v>
       </c>
-      <c r="M13" s="8">
+      <c r="M13" s="7">
         <v>6.2239999999999997E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:13" s="4" customFormat="1">
+    <row r="14" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -1272,7 +1072,7 @@
         <v>-0.12891</v>
       </c>
     </row>
-    <row r="15" spans="1:13" s="4" customFormat="1">
+    <row r="15" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>1</v>
       </c>
@@ -1313,7 +1113,7 @@
         <v>0.36362</v>
       </c>
     </row>
-    <row r="16" spans="1:13" s="4" customFormat="1">
+    <row r="16" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>1</v>
       </c>
@@ -1354,7 +1154,7 @@
         <v>0.10390000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:13" s="4" customFormat="1">
+    <row r="17" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>1</v>
       </c>
@@ -1395,7 +1195,7 @@
         <v>-3.4410000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" s="4" customFormat="1">
+    <row r="18" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>1</v>
       </c>
@@ -1436,7 +1236,7 @@
         <v>1.8579999999999999E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:13" s="4" customFormat="1">
+    <row r="19" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>1</v>
       </c>
@@ -1477,7 +1277,7 @@
         <v>-4.2799999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:13" s="4" customFormat="1">
+    <row r="20" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>1</v>
       </c>
@@ -1518,7 +1318,7 @@
         <v>-0.23998</v>
       </c>
     </row>
-    <row r="21" spans="1:13" s="4" customFormat="1">
+    <row r="21" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>1</v>
       </c>
@@ -1559,7 +1359,7 @@
         <v>-0.2213</v>
       </c>
     </row>
-    <row r="22" spans="1:13" s="4" customFormat="1">
+    <row r="22" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>1</v>
       </c>
@@ -1600,7 +1400,7 @@
         <v>-0.32107000000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:13" s="4" customFormat="1">
+    <row r="23" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>1</v>
       </c>
@@ -1641,7 +1441,7 @@
         <v>-0.49713000000000002</v>
       </c>
     </row>
-    <row r="24" spans="1:13" s="4" customFormat="1">
+    <row r="24" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>1</v>
       </c>
@@ -1682,7 +1482,7 @@
         <v>-0.43210999999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:13" s="4" customFormat="1">
+    <row r="25" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>1</v>
       </c>
@@ -1723,7 +1523,7 @@
         <v>-0.34375</v>
       </c>
     </row>
-    <row r="26" spans="1:13" s="4" customFormat="1">
+    <row r="26" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>1</v>
       </c>
@@ -1764,7 +1564,7 @@
         <v>-0.41450999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:13" s="4" customFormat="1">
+    <row r="27" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>1</v>
       </c>
@@ -1805,7 +1605,7 @@
         <v>-0.41563</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>1</v>
       </c>
@@ -1846,1864 +1646,1864 @@
         <v>-0.38588</v>
       </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B29" s="12">
+      <c r="B29" s="11">
         <v>-1.2083999999999999</v>
       </c>
-      <c r="C29" s="12">
+      <c r="C29" s="11">
         <v>1.2352799999999999</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="11">
         <v>-0.71531999999999996</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="11">
         <v>-1.1348400000000001</v>
       </c>
-      <c r="F29" s="12">
+      <c r="F29" s="11">
         <v>-0.32958999999999999</v>
       </c>
-      <c r="G29" s="13">
+      <c r="G29" s="12">
         <v>0.87817999999999996</v>
       </c>
-      <c r="H29" s="12">
+      <c r="H29" s="11">
         <v>-1.10131</v>
       </c>
-      <c r="I29" s="12">
+      <c r="I29" s="11">
         <v>-0.18883</v>
       </c>
-      <c r="J29" s="12">
+      <c r="J29" s="11">
         <v>-3.1579999999999997E-2</v>
       </c>
-      <c r="K29" s="12">
+      <c r="K29" s="11">
         <v>2.2745700000000002</v>
       </c>
-      <c r="L29" s="12">
+      <c r="L29" s="11">
         <v>-0.47336</v>
       </c>
-      <c r="M29" s="12">
+      <c r="M29" s="11">
         <v>-0.24510000000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B30" s="12">
+      <c r="B30" s="11">
         <v>-1.22922</v>
       </c>
-      <c r="C30" s="12">
+      <c r="C30" s="11">
         <v>1.1311800000000001</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="11">
         <v>-1.00522</v>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="11">
         <v>-1.3686199999999999</v>
       </c>
-      <c r="F30" s="12">
+      <c r="F30" s="11">
         <v>1.736E-2</v>
       </c>
-      <c r="G30" s="13">
+      <c r="G30" s="12">
         <v>0.73768</v>
       </c>
-      <c r="H30" s="12">
+      <c r="H30" s="11">
         <v>-1.18655</v>
       </c>
-      <c r="I30" s="12">
+      <c r="I30" s="11">
         <v>-0.27173999999999998</v>
       </c>
-      <c r="J30" s="12">
+      <c r="J30" s="11">
         <v>-0.18110999999999999</v>
       </c>
-      <c r="K30" s="12">
+      <c r="K30" s="11">
         <v>2.5556700000000001</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L30" s="11">
         <v>-0.18981999999999999</v>
       </c>
-      <c r="M30" s="12">
+      <c r="M30" s="11">
         <v>-0.24629999999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B31" s="12">
+      <c r="B31" s="11">
         <v>-0.94613000000000003</v>
       </c>
-      <c r="C31" s="12">
+      <c r="C31" s="11">
         <v>1.5626899999999999</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="11">
         <v>-0.21631</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="11">
         <v>-1.1076900000000001</v>
       </c>
-      <c r="F31" s="12">
+      <c r="F31" s="11">
         <v>0.18626999999999999</v>
       </c>
-      <c r="G31" s="13">
+      <c r="G31" s="12">
         <v>0.74480000000000002</v>
       </c>
-      <c r="H31" s="12">
+      <c r="H31" s="11">
         <v>-0.72624</v>
       </c>
-      <c r="I31" s="12">
+      <c r="I31" s="11">
         <v>-0.45101999999999998</v>
       </c>
-      <c r="J31" s="12">
+      <c r="J31" s="11">
         <v>2.3480000000000001E-2</v>
       </c>
-      <c r="K31" s="12">
+      <c r="K31" s="11">
         <v>1.4542900000000001</v>
       </c>
-      <c r="L31" s="12">
+      <c r="L31" s="11">
         <v>-0.30375000000000002</v>
       </c>
-      <c r="M31" s="12">
+      <c r="M31" s="11">
         <v>-0.21811</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B32" s="12">
+      <c r="B32" s="11">
         <v>-0.69503999999999999</v>
       </c>
-      <c r="C32" s="12">
+      <c r="C32" s="11">
         <v>2.0990600000000001</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="11">
         <v>8.7059999999999998E-2</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="11">
         <v>-0.59680999999999995</v>
       </c>
-      <c r="F32" s="12">
+      <c r="F32" s="11">
         <v>0.42318</v>
       </c>
-      <c r="G32" s="13">
+      <c r="G32" s="12">
         <v>1.2300500000000001</v>
       </c>
-      <c r="H32" s="12">
+      <c r="H32" s="11">
         <v>-0.70218999999999998</v>
       </c>
-      <c r="I32" s="12">
+      <c r="I32" s="11">
         <v>-0.45713999999999999</v>
       </c>
-      <c r="J32" s="12">
+      <c r="J32" s="11">
         <v>0.30420000000000003</v>
       </c>
-      <c r="K32" s="12">
+      <c r="K32" s="11">
         <v>1.4106300000000001</v>
       </c>
-      <c r="L32" s="12">
+      <c r="L32" s="11">
         <v>-0.37645000000000001</v>
       </c>
-      <c r="M32" s="12">
+      <c r="M32" s="11">
         <v>-0.13922000000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B33" s="12">
+      <c r="B33" s="11">
         <v>-1.3241000000000001</v>
       </c>
-      <c r="C33" s="12">
+      <c r="C33" s="11">
         <v>1.9882899999999999</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="11">
         <v>-0.26128000000000001</v>
       </c>
-      <c r="E33" s="12">
+      <c r="E33" s="11">
         <v>-0.71528999999999998</v>
       </c>
-      <c r="F33" s="12">
+      <c r="F33" s="11">
         <v>0.28905999999999998</v>
       </c>
-      <c r="G33" s="13">
+      <c r="G33" s="12">
         <v>0.75521000000000005</v>
       </c>
-      <c r="H33" s="12">
+      <c r="H33" s="11">
         <v>-1.3332999999999999</v>
       </c>
-      <c r="I33" s="12">
+      <c r="I33" s="11">
         <v>-0.33825</v>
       </c>
-      <c r="J33" s="12">
+      <c r="J33" s="11">
         <v>-8.0210000000000004E-2</v>
       </c>
-      <c r="K33" s="12">
+      <c r="K33" s="11">
         <v>1.72444</v>
       </c>
-      <c r="L33" s="12">
+      <c r="L33" s="11">
         <v>-0.33254</v>
       </c>
-      <c r="M33" s="12">
+      <c r="M33" s="11">
         <v>-0.28497</v>
       </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B34" s="12">
+      <c r="B34" s="11">
         <v>-1.4680599999999999</v>
       </c>
-      <c r="C34" s="12">
+      <c r="C34" s="11">
         <v>1.71753</v>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="11">
         <v>-1.09598</v>
       </c>
-      <c r="E34" s="12">
+      <c r="E34" s="11">
         <v>-1.11009</v>
       </c>
-      <c r="F34" s="12">
+      <c r="F34" s="11">
         <v>5.1049999999999998E-2</v>
       </c>
-      <c r="G34" s="13">
+      <c r="G34" s="12">
         <v>0.63202999999999998</v>
       </c>
-      <c r="H34" s="12">
+      <c r="H34" s="11">
         <v>-1.57125</v>
       </c>
-      <c r="I34" s="12">
+      <c r="I34" s="11">
         <v>-0.41792000000000001</v>
       </c>
-      <c r="J34" s="12">
+      <c r="J34" s="11">
         <v>-0.17868999999999999</v>
       </c>
-      <c r="K34" s="12">
+      <c r="K34" s="11">
         <v>2.2224699999999999</v>
       </c>
-      <c r="L34" s="12">
+      <c r="L34" s="11">
         <v>-0.23222000000000001</v>
       </c>
-      <c r="M34" s="12">
+      <c r="M34" s="11">
         <v>-0.30756</v>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B35" s="12">
+      <c r="B35" s="11">
         <v>-1.1748499999999999</v>
       </c>
-      <c r="C35" s="12">
+      <c r="C35" s="11">
         <v>1.4761299999999999</v>
       </c>
-      <c r="D35" s="12">
+      <c r="D35" s="11">
         <v>-0.47350999999999999</v>
       </c>
-      <c r="E35" s="12">
+      <c r="E35" s="11">
         <v>-1.11046</v>
       </c>
-      <c r="F35" s="12">
+      <c r="F35" s="11">
         <v>0.26125999999999999</v>
       </c>
-      <c r="G35" s="13">
+      <c r="G35" s="12">
         <v>0.58538000000000001</v>
       </c>
-      <c r="H35" s="12">
+      <c r="H35" s="11">
         <v>-1.12276</v>
       </c>
-      <c r="I35" s="12">
+      <c r="I35" s="11">
         <v>-0.27582000000000001</v>
       </c>
-      <c r="J35" s="12">
+      <c r="J35" s="11">
         <v>0.12417</v>
       </c>
-      <c r="K35" s="12">
+      <c r="K35" s="11">
         <v>1.77888</v>
       </c>
-      <c r="L35" s="12">
+      <c r="L35" s="11">
         <v>-0.33561000000000002</v>
       </c>
-      <c r="M35" s="12">
+      <c r="M35" s="11">
         <v>-0.13908999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B36" s="12">
+      <c r="B36" s="11">
         <v>-1.11957</v>
       </c>
-      <c r="C36" s="12">
+      <c r="C36" s="11">
         <v>1.6997599999999999</v>
       </c>
-      <c r="D36" s="12">
+      <c r="D36" s="11">
         <v>-0.40669</v>
       </c>
-      <c r="E36" s="12">
+      <c r="E36" s="11">
         <v>-0.87021999999999999</v>
       </c>
-      <c r="F36" s="12">
+      <c r="F36" s="11">
         <v>0.28193000000000001</v>
       </c>
-      <c r="G36" s="13">
+      <c r="G36" s="12">
         <v>0.60611999999999999</v>
       </c>
-      <c r="H36" s="12">
+      <c r="H36" s="11">
         <v>-1.03685</v>
       </c>
-      <c r="I36" s="12">
+      <c r="I36" s="11">
         <v>-0.30754999999999999</v>
       </c>
-      <c r="J36" s="12">
+      <c r="J36" s="11">
         <v>9.2179999999999998E-2</v>
       </c>
-      <c r="K36" s="12">
+      <c r="K36" s="11">
         <v>1.6114299999999999</v>
       </c>
-      <c r="L36" s="12">
+      <c r="L36" s="11">
         <v>-0.47638000000000003</v>
       </c>
-      <c r="M36" s="12">
+      <c r="M36" s="11">
         <v>-0.20866999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B37" s="12">
+      <c r="B37" s="11">
         <v>-1.1451199999999999</v>
       </c>
-      <c r="C37" s="12">
+      <c r="C37" s="11">
         <v>1.50075</v>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="11">
         <v>-0.57738</v>
       </c>
-      <c r="E37" s="12">
+      <c r="E37" s="11">
         <v>-1.0672699999999999</v>
       </c>
-      <c r="F37" s="12">
+      <c r="F37" s="11">
         <v>-0.10653</v>
       </c>
-      <c r="G37" s="13">
+      <c r="G37" s="12">
         <v>0.61477999999999999</v>
       </c>
-      <c r="H37" s="12">
+      <c r="H37" s="11">
         <v>-1.33666</v>
       </c>
-      <c r="I37" s="12">
+      <c r="I37" s="11">
         <v>-0.22048999999999999</v>
       </c>
-      <c r="J37" s="12">
+      <c r="J37" s="11">
         <v>0.51119999999999999</v>
       </c>
-      <c r="K37" s="12">
+      <c r="K37" s="11">
         <v>1.2170399999999999</v>
       </c>
-      <c r="L37" s="12">
+      <c r="L37" s="11">
         <v>-0.13880000000000001</v>
       </c>
-      <c r="M37" s="12">
+      <c r="M37" s="11">
         <v>-0.31235000000000002</v>
       </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B38" s="12">
+      <c r="B38" s="11">
         <v>-1.06541</v>
       </c>
-      <c r="C38" s="12">
+      <c r="C38" s="11">
         <v>1.63192</v>
       </c>
-      <c r="D38" s="12">
+      <c r="D38" s="11">
         <v>-0.44180999999999998</v>
       </c>
-      <c r="E38" s="12">
+      <c r="E38" s="11">
         <v>-0.68652000000000002</v>
       </c>
-      <c r="F38" s="12">
+      <c r="F38" s="11">
         <v>0.31536999999999998</v>
       </c>
-      <c r="G38" s="13">
+      <c r="G38" s="12">
         <v>0.90956999999999999</v>
       </c>
-      <c r="H38" s="12">
+      <c r="H38" s="11">
         <v>-1.3687100000000001</v>
       </c>
-      <c r="I38" s="12">
+      <c r="I38" s="11">
         <v>-0.31591999999999998</v>
       </c>
-      <c r="J38" s="12">
+      <c r="J38" s="11">
         <v>0.72940000000000005</v>
       </c>
-      <c r="K38" s="12">
+      <c r="K38" s="11">
         <v>1.35388</v>
       </c>
-      <c r="L38" s="12">
+      <c r="L38" s="11">
         <v>-0.26573000000000002</v>
       </c>
-      <c r="M38" s="12">
+      <c r="M38" s="11">
         <v>-0.19114999999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B39" s="12">
+      <c r="B39" s="11">
         <v>-1.0145599999999999</v>
       </c>
-      <c r="C39" s="12">
+      <c r="C39" s="11">
         <v>1.8247100000000001</v>
       </c>
-      <c r="D39" s="12">
+      <c r="D39" s="11">
         <v>-0.34366999999999998</v>
       </c>
-      <c r="E39" s="12">
+      <c r="E39" s="11">
         <v>-0.75348999999999999</v>
       </c>
-      <c r="F39" s="12">
+      <c r="F39" s="11">
         <v>0.29581000000000002</v>
       </c>
-      <c r="G39" s="13">
+      <c r="G39" s="12">
         <v>1.11954</v>
       </c>
-      <c r="H39" s="12">
+      <c r="H39" s="11">
         <v>-1.2730399999999999</v>
       </c>
-      <c r="I39" s="12">
+      <c r="I39" s="11">
         <v>-0.46</v>
       </c>
-      <c r="J39" s="12">
+      <c r="J39" s="11">
         <v>0.14321999999999999</v>
       </c>
-      <c r="K39" s="12">
+      <c r="K39" s="11">
         <v>1.78315</v>
       </c>
-      <c r="L39" s="12">
+      <c r="L39" s="11">
         <v>-0.44283</v>
       </c>
-      <c r="M39" s="12">
+      <c r="M39" s="11">
         <v>-0.26982</v>
       </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B40" s="12">
+      <c r="B40" s="11">
         <v>-0.96314999999999995</v>
       </c>
-      <c r="C40" s="12">
+      <c r="C40" s="11">
         <v>1.48722</v>
       </c>
-      <c r="D40" s="12">
+      <c r="D40" s="11">
         <v>-0.40483000000000002</v>
       </c>
-      <c r="E40" s="12">
+      <c r="E40" s="11">
         <v>-1.0572900000000001</v>
       </c>
-      <c r="F40" s="12">
+      <c r="F40" s="11">
         <v>0.31053999999999998</v>
       </c>
-      <c r="G40" s="13">
+      <c r="G40" s="12">
         <v>0.94404999999999994</v>
       </c>
-      <c r="H40" s="12">
+      <c r="H40" s="11">
         <v>-0.77400000000000002</v>
       </c>
-      <c r="I40" s="12">
+      <c r="I40" s="11">
         <v>-0.19167999999999999</v>
       </c>
-      <c r="J40" s="12">
+      <c r="J40" s="11">
         <v>0.23351</v>
       </c>
-      <c r="K40" s="12">
+      <c r="K40" s="11">
         <v>1.6425700000000001</v>
       </c>
-      <c r="L40" s="12">
+      <c r="L40" s="11">
         <v>-0.53363000000000005</v>
       </c>
-      <c r="M40" s="12">
+      <c r="M40" s="11">
         <v>-0.12716</v>
       </c>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B41" s="12">
+      <c r="B41" s="11">
         <v>-0.63161</v>
       </c>
-      <c r="C41" s="12">
+      <c r="C41" s="11">
         <v>1.86853</v>
       </c>
-      <c r="D41" s="12">
+      <c r="D41" s="11">
         <v>0.19464000000000001</v>
       </c>
-      <c r="E41" s="12">
+      <c r="E41" s="11">
         <v>-0.60221000000000002</v>
       </c>
-      <c r="F41" s="12">
+      <c r="F41" s="11">
         <v>0.45307999999999998</v>
       </c>
-      <c r="G41" s="13">
+      <c r="G41" s="12">
         <v>1.4004700000000001</v>
       </c>
-      <c r="H41" s="12">
+      <c r="H41" s="11">
         <v>-0.97792999999999997</v>
       </c>
-      <c r="I41" s="12">
+      <c r="I41" s="11">
         <v>-0.42316999999999999</v>
       </c>
-      <c r="J41" s="12">
+      <c r="J41" s="11">
         <v>0.51002000000000003</v>
       </c>
-      <c r="K41" s="12">
+      <c r="K41" s="11">
         <v>2.0363799999999999</v>
       </c>
-      <c r="L41" s="12">
+      <c r="L41" s="11">
         <v>-0.48398999999999998</v>
       </c>
-      <c r="M41" s="12">
+      <c r="M41" s="11">
         <v>-0.14248</v>
       </c>
     </row>
-    <row r="42" spans="1:13">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B42" s="12">
+      <c r="B42" s="11">
         <v>-1.18218</v>
       </c>
-      <c r="C42" s="12">
+      <c r="C42" s="11">
         <v>1.12557</v>
       </c>
-      <c r="D42" s="12">
+      <c r="D42" s="11">
         <v>-0.71718999999999999</v>
       </c>
-      <c r="E42" s="12">
+      <c r="E42" s="11">
         <v>-1.10965</v>
       </c>
-      <c r="F42" s="12">
+      <c r="F42" s="11">
         <v>0.12035999999999999</v>
       </c>
-      <c r="G42" s="13">
+      <c r="G42" s="12">
         <v>0.70986000000000005</v>
       </c>
-      <c r="H42" s="12">
+      <c r="H42" s="11">
         <v>-1.4820599999999999</v>
       </c>
-      <c r="I42" s="12">
+      <c r="I42" s="11">
         <v>0.13533000000000001</v>
       </c>
-      <c r="J42" s="12">
+      <c r="J42" s="11">
         <v>0.27877999999999997</v>
       </c>
-      <c r="K42" s="12">
+      <c r="K42" s="11">
         <v>2.5474299999999999</v>
       </c>
-      <c r="L42" s="12">
+      <c r="L42" s="11">
         <v>-0.31564999999999999</v>
       </c>
-      <c r="M42" s="12">
+      <c r="M42" s="11">
         <v>-0.18806</v>
       </c>
     </row>
-    <row r="43" spans="1:13">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B43" s="12">
+      <c r="B43" s="11">
         <v>-0.82169999999999999</v>
       </c>
-      <c r="C43" s="12">
+      <c r="C43" s="11">
         <v>1.7338499999999999</v>
       </c>
-      <c r="D43" s="12">
+      <c r="D43" s="11">
         <v>-0.47008</v>
       </c>
-      <c r="E43" s="12">
+      <c r="E43" s="11">
         <v>-1.0249600000000001</v>
       </c>
-      <c r="F43" s="12">
+      <c r="F43" s="11">
         <v>0.1736</v>
       </c>
-      <c r="G43" s="13">
+      <c r="G43" s="12">
         <v>0.79713999999999996</v>
       </c>
-      <c r="H43" s="12">
+      <c r="H43" s="11">
         <v>-1.2452099999999999</v>
       </c>
-      <c r="I43" s="12">
+      <c r="I43" s="11">
         <v>-0.31494</v>
       </c>
-      <c r="J43" s="12">
+      <c r="J43" s="11">
         <v>0.31359999999999999</v>
       </c>
-      <c r="K43" s="12">
+      <c r="K43" s="11">
         <v>2.2482799999999998</v>
       </c>
-      <c r="L43" s="12">
+      <c r="L43" s="11">
         <v>-0.24886</v>
       </c>
-      <c r="M43" s="12">
+      <c r="M43" s="11">
         <v>-0.22173000000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B44" s="12">
+      <c r="B44" s="11">
         <v>-1.06816</v>
       </c>
-      <c r="C44" s="12">
+      <c r="C44" s="11">
         <v>1.59476</v>
       </c>
-      <c r="D44" s="12">
+      <c r="D44" s="11">
         <v>-0.49431999999999998</v>
       </c>
-      <c r="E44" s="12">
+      <c r="E44" s="11">
         <v>-0.75219000000000003</v>
       </c>
-      <c r="F44" s="12">
+      <c r="F44" s="11">
         <v>0.25952999999999998</v>
       </c>
-      <c r="G44" s="13">
+      <c r="G44" s="12">
         <v>0.70992</v>
       </c>
-      <c r="H44" s="12">
+      <c r="H44" s="11">
         <v>-1.4914799999999999</v>
       </c>
-      <c r="I44" s="12">
+      <c r="I44" s="11">
         <v>-0.18281</v>
       </c>
-      <c r="J44" s="12">
+      <c r="J44" s="11">
         <v>-1.8579999999999999E-2</v>
       </c>
-      <c r="K44" s="12">
+      <c r="K44" s="11">
         <v>1.84633</v>
       </c>
-      <c r="L44" s="12">
+      <c r="L44" s="11">
         <v>-0.3831</v>
       </c>
-      <c r="M44" s="12">
+      <c r="M44" s="11">
         <v>-0.35181000000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:13">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B45" s="12">
+      <c r="B45" s="11">
         <v>-1.1783999999999999</v>
       </c>
-      <c r="C45" s="12">
+      <c r="C45" s="11">
         <v>1.0932200000000001</v>
       </c>
-      <c r="D45" s="12">
+      <c r="D45" s="11">
         <v>-0.48797000000000001</v>
       </c>
-      <c r="E45" s="12">
+      <c r="E45" s="11">
         <v>-1.19163</v>
       </c>
-      <c r="F45" s="12">
+      <c r="F45" s="11">
         <v>0.14280000000000001</v>
       </c>
-      <c r="G45" s="13">
+      <c r="G45" s="12">
         <v>0.97653000000000001</v>
       </c>
-      <c r="H45" s="12">
+      <c r="H45" s="11">
         <v>-1.5720099999999999</v>
       </c>
-      <c r="I45" s="12">
+      <c r="I45" s="11">
         <v>-0.12823000000000001</v>
       </c>
-      <c r="J45" s="12">
+      <c r="J45" s="11">
         <v>5.101E-2</v>
       </c>
-      <c r="K45" s="12">
+      <c r="K45" s="11">
         <v>2.7487400000000002</v>
       </c>
-      <c r="L45" s="12">
+      <c r="L45" s="11">
         <v>-0.27567000000000003</v>
       </c>
-      <c r="M45" s="12">
+      <c r="M45" s="11">
         <v>-0.36004999999999998</v>
       </c>
     </row>
-    <row r="46" spans="1:13">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B46" s="12">
+      <c r="B46" s="11">
         <v>-1.0864100000000001</v>
       </c>
-      <c r="C46" s="12">
+      <c r="C46" s="11">
         <v>1.53769</v>
       </c>
-      <c r="D46" s="12">
+      <c r="D46" s="11">
         <v>-0.35320000000000001</v>
       </c>
-      <c r="E46" s="12">
+      <c r="E46" s="11">
         <v>-0.75329999999999997</v>
       </c>
-      <c r="F46" s="12">
+      <c r="F46" s="11">
         <v>0.33706999999999998</v>
       </c>
-      <c r="G46" s="13">
+      <c r="G46" s="12">
         <v>0.87129999999999996</v>
       </c>
-      <c r="H46" s="12">
+      <c r="H46" s="11">
         <v>-1.38297</v>
       </c>
-      <c r="I46" s="12">
+      <c r="I46" s="11">
         <v>-0.20097000000000001</v>
       </c>
-      <c r="J46" s="12">
+      <c r="J46" s="11">
         <v>0.36371999999999999</v>
       </c>
-      <c r="K46" s="12">
+      <c r="K46" s="11">
         <v>1.90002</v>
       </c>
-      <c r="L46" s="12">
+      <c r="L46" s="11">
         <v>-0.39494000000000001</v>
       </c>
-      <c r="M46" s="12">
+      <c r="M46" s="11">
         <v>-0.33035999999999999</v>
       </c>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B47" s="12">
+      <c r="B47" s="11">
         <v>-1.27504</v>
       </c>
-      <c r="C47" s="12">
+      <c r="C47" s="11">
         <v>1.61056</v>
       </c>
-      <c r="D47" s="12">
+      <c r="D47" s="11">
         <v>-1.1573500000000001</v>
       </c>
-      <c r="E47" s="12">
+      <c r="E47" s="11">
         <v>-1.23837</v>
       </c>
-      <c r="F47" s="12">
+      <c r="F47" s="11">
         <v>0.1532</v>
       </c>
-      <c r="G47" s="13">
+      <c r="G47" s="12">
         <v>0.44252999999999998</v>
       </c>
-      <c r="H47" s="12">
+      <c r="H47" s="11">
         <v>-1.40662</v>
       </c>
-      <c r="I47" s="12">
+      <c r="I47" s="11">
         <v>-0.3669</v>
       </c>
-      <c r="J47" s="12">
+      <c r="J47" s="11">
         <v>0.17224999999999999</v>
       </c>
-      <c r="K47" s="12">
+      <c r="K47" s="11">
         <v>1.98004</v>
       </c>
-      <c r="L47" s="12">
+      <c r="L47" s="11">
         <v>-0.35621999999999998</v>
       </c>
-      <c r="M47" s="12">
+      <c r="M47" s="11">
         <v>-0.40303</v>
       </c>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B48" s="12">
+      <c r="B48" s="11">
         <v>-1.16204</v>
       </c>
-      <c r="C48" s="12">
+      <c r="C48" s="11">
         <v>1.49169</v>
       </c>
-      <c r="D48" s="12">
+      <c r="D48" s="11">
         <v>-0.55274000000000001</v>
       </c>
-      <c r="E48" s="12">
+      <c r="E48" s="11">
         <v>-0.84509999999999996</v>
       </c>
-      <c r="F48" s="12">
+      <c r="F48" s="11">
         <v>0.23526</v>
       </c>
-      <c r="G48" s="13">
+      <c r="G48" s="12">
         <v>0.71057000000000003</v>
       </c>
-      <c r="H48" s="12">
+      <c r="H48" s="11">
         <v>-1.62808</v>
       </c>
-      <c r="I48" s="12">
+      <c r="I48" s="11">
         <v>-1.788E-2</v>
       </c>
-      <c r="J48" s="12">
+      <c r="J48" s="11">
         <v>0.33331</v>
       </c>
-      <c r="K48" s="12">
+      <c r="K48" s="11">
         <v>2.02685</v>
       </c>
-      <c r="L48" s="12">
+      <c r="L48" s="11">
         <v>-0.39595999999999998</v>
       </c>
-      <c r="M48" s="12">
+      <c r="M48" s="11">
         <v>-0.28720000000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:13">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B49" s="12">
+      <c r="B49" s="11">
         <v>-1.05474</v>
       </c>
-      <c r="C49" s="12">
+      <c r="C49" s="11">
         <v>1.2202500000000001</v>
       </c>
-      <c r="D49" s="12">
+      <c r="D49" s="11">
         <v>-0.71267999999999998</v>
       </c>
-      <c r="E49" s="12">
+      <c r="E49" s="11">
         <v>-1.1363700000000001</v>
       </c>
-      <c r="F49" s="12">
+      <c r="F49" s="11">
         <v>0.26416000000000001</v>
       </c>
-      <c r="G49" s="13">
+      <c r="G49" s="12">
         <v>0.73926000000000003</v>
       </c>
-      <c r="H49" s="12">
+      <c r="H49" s="11">
         <v>-1.33325</v>
       </c>
-      <c r="I49" s="12">
+      <c r="I49" s="11">
         <v>-0.28577000000000002</v>
       </c>
-      <c r="J49" s="12">
+      <c r="J49" s="11">
         <v>0.24822</v>
       </c>
-      <c r="K49" s="12">
+      <c r="K49" s="11">
         <v>2.4430999999999998</v>
       </c>
-      <c r="L49" s="12">
+      <c r="L49" s="11">
         <v>-0.31785000000000002</v>
       </c>
-      <c r="M49" s="12">
+      <c r="M49" s="11">
         <v>-0.21731</v>
       </c>
     </row>
-    <row r="50" spans="1:13">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B50" s="12">
+      <c r="B50" s="11">
         <v>-0.89812000000000003</v>
       </c>
-      <c r="C50" s="12">
+      <c r="C50" s="11">
         <v>1.5566500000000001</v>
       </c>
-      <c r="D50" s="12">
+      <c r="D50" s="11">
         <v>-0.41810999999999998</v>
       </c>
-      <c r="E50" s="12">
+      <c r="E50" s="11">
         <v>-1.0066600000000001</v>
       </c>
-      <c r="F50" s="12">
+      <c r="F50" s="11">
         <v>0.23608000000000001</v>
       </c>
-      <c r="G50" s="13">
+      <c r="G50" s="12">
         <v>0.98697999999999997</v>
       </c>
-      <c r="H50" s="12">
+      <c r="H50" s="11">
         <v>-1.1273500000000001</v>
       </c>
-      <c r="I50" s="12">
+      <c r="I50" s="11">
         <v>-0.49413000000000001</v>
       </c>
-      <c r="J50" s="12">
+      <c r="J50" s="11">
         <v>9.3700000000000006E-2</v>
       </c>
-      <c r="K50" s="12">
+      <c r="K50" s="11">
         <v>2.1270899999999999</v>
       </c>
-      <c r="L50" s="12">
+      <c r="L50" s="11">
         <v>-0.38144</v>
       </c>
-      <c r="M50" s="12">
+      <c r="M50" s="11">
         <v>-0.35458000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:13">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B51" s="12">
+      <c r="B51" s="11">
         <v>-1.2175</v>
       </c>
-      <c r="C51" s="12">
+      <c r="C51" s="11">
         <v>2.07335</v>
       </c>
-      <c r="D51" s="12">
+      <c r="D51" s="11">
         <v>-0.12024</v>
       </c>
-      <c r="E51" s="12">
+      <c r="E51" s="11">
         <v>-0.70916999999999997</v>
       </c>
-      <c r="F51" s="12">
+      <c r="F51" s="11">
         <v>0.31714999999999999</v>
       </c>
-      <c r="G51" s="13">
+      <c r="G51" s="12">
         <v>0.69418999999999997</v>
       </c>
-      <c r="H51" s="12">
+      <c r="H51" s="11">
         <v>-0.66805999999999999</v>
       </c>
-      <c r="I51" s="12">
+      <c r="I51" s="11">
         <v>-0.56637999999999999</v>
       </c>
-      <c r="J51" s="12">
+      <c r="J51" s="11">
         <v>0.25722</v>
       </c>
-      <c r="K51" s="12">
+      <c r="K51" s="11">
         <v>0.8861</v>
       </c>
-      <c r="L51" s="12">
+      <c r="L51" s="11">
         <v>-0.66325000000000001</v>
       </c>
-      <c r="M51" s="12">
+      <c r="M51" s="11">
         <v>-0.28621999999999997</v>
       </c>
     </row>
-    <row r="52" spans="1:13">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B52" s="12">
+      <c r="B52" s="11">
         <v>-0.91959000000000002</v>
       </c>
-      <c r="C52" s="12">
+      <c r="C52" s="11">
         <v>1.34328</v>
       </c>
-      <c r="D52" s="12">
+      <c r="D52" s="11">
         <v>-0.29785</v>
       </c>
-      <c r="E52" s="12">
+      <c r="E52" s="11">
         <v>-0.96106999999999998</v>
       </c>
-      <c r="F52" s="12">
+      <c r="F52" s="11">
         <v>0.38612000000000002</v>
       </c>
-      <c r="G52" s="13">
+      <c r="G52" s="12">
         <v>1.0182800000000001</v>
       </c>
-      <c r="H52" s="12">
+      <c r="H52" s="11">
         <v>-1.23383</v>
       </c>
-      <c r="I52" s="12">
+      <c r="I52" s="11">
         <v>-2.4049999999999998E-2</v>
       </c>
-      <c r="J52" s="12">
+      <c r="J52" s="11">
         <v>0.35155999999999998</v>
       </c>
-      <c r="K52" s="12">
+      <c r="K52" s="11">
         <v>2.3641200000000002</v>
       </c>
-      <c r="L52" s="12">
+      <c r="L52" s="11">
         <v>-0.38159999999999999</v>
       </c>
-      <c r="M52" s="12">
+      <c r="M52" s="11">
         <v>-0.22464000000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:13">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B53" s="12">
+      <c r="B53" s="11">
         <v>-1.3594999999999999</v>
       </c>
-      <c r="C53" s="12">
+      <c r="C53" s="11">
         <v>1.4438800000000001</v>
       </c>
-      <c r="D53" s="12">
+      <c r="D53" s="11">
         <v>-0.62727999999999995</v>
       </c>
-      <c r="E53" s="12">
+      <c r="E53" s="11">
         <v>-0.91842999999999997</v>
       </c>
-      <c r="F53" s="12">
+      <c r="F53" s="11">
         <v>0.19836000000000001</v>
       </c>
-      <c r="G53" s="13">
+      <c r="G53" s="12">
         <v>0.58357999999999999</v>
       </c>
-      <c r="H53" s="12">
+      <c r="H53" s="11">
         <v>-1.1358200000000001</v>
       </c>
-      <c r="I53" s="12">
+      <c r="I53" s="11">
         <v>-0.16575000000000001</v>
       </c>
-      <c r="J53" s="12">
+      <c r="J53" s="11">
         <v>0.25895000000000001</v>
       </c>
-      <c r="K53" s="12">
+      <c r="K53" s="11">
         <v>1.36541</v>
       </c>
-      <c r="L53" s="12">
+      <c r="L53" s="11">
         <v>-0.40958</v>
       </c>
-      <c r="M53" s="12">
+      <c r="M53" s="11">
         <v>-0.24804000000000001</v>
       </c>
     </row>
-    <row r="54" spans="1:13">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B54" s="12">
+      <c r="B54" s="11">
         <v>-0.89571999999999996</v>
       </c>
-      <c r="C54" s="12">
+      <c r="C54" s="11">
         <v>1.8649</v>
       </c>
-      <c r="D54" s="12">
+      <c r="D54" s="11">
         <v>-0.24401999999999999</v>
       </c>
-      <c r="E54" s="12">
+      <c r="E54" s="11">
         <v>-0.86006000000000005</v>
       </c>
-      <c r="F54" s="12">
+      <c r="F54" s="11">
         <v>0.42913000000000001</v>
       </c>
-      <c r="G54" s="13">
+      <c r="G54" s="12">
         <v>0.95538999999999996</v>
       </c>
-      <c r="H54" s="12">
+      <c r="H54" s="11">
         <v>-0.97829999999999995</v>
       </c>
-      <c r="I54" s="12">
+      <c r="I54" s="11">
         <v>-0.28028999999999998</v>
       </c>
-      <c r="J54" s="12">
+      <c r="J54" s="11">
         <v>0.26055</v>
       </c>
-      <c r="K54" s="12">
+      <c r="K54" s="11">
         <v>2.0491799999999998</v>
       </c>
-      <c r="L54" s="12">
+      <c r="L54" s="11">
         <v>-0.34964000000000001</v>
       </c>
-      <c r="M54" s="12">
+      <c r="M54" s="11">
         <v>-0.17927999999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:13">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B55" s="12">
+      <c r="B55" s="11">
         <v>-1.5230399999999999</v>
       </c>
-      <c r="C55" s="12">
+      <c r="C55" s="11">
         <v>1.47163</v>
       </c>
-      <c r="D55" s="12">
+      <c r="D55" s="11">
         <v>-1.2669999999999999</v>
       </c>
-      <c r="E55" s="12">
+      <c r="E55" s="11">
         <v>-1.3667100000000001</v>
       </c>
-      <c r="F55" s="12">
+      <c r="F55" s="11">
         <v>0.11515</v>
       </c>
-      <c r="G55" s="13">
+      <c r="G55" s="12">
         <v>0.27787000000000001</v>
       </c>
-      <c r="H55" s="12">
+      <c r="H55" s="11">
         <v>-1.17997</v>
       </c>
-      <c r="I55" s="12">
+      <c r="I55" s="11">
         <v>-0.45544000000000001</v>
       </c>
-      <c r="J55" s="12">
+      <c r="J55" s="11">
         <v>-0.11458</v>
       </c>
-      <c r="K55" s="12">
+      <c r="K55" s="11">
         <v>1.7778</v>
       </c>
-      <c r="L55" s="12">
+      <c r="L55" s="11">
         <v>-0.26758999999999999</v>
       </c>
-      <c r="M55" s="12">
+      <c r="M55" s="11">
         <v>-0.28763</v>
       </c>
     </row>
-    <row r="56" spans="1:13">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B56" s="12">
+      <c r="B56" s="11">
         <v>-1.0745899999999999</v>
       </c>
-      <c r="C56" s="12">
+      <c r="C56" s="11">
         <v>1.2802800000000001</v>
       </c>
-      <c r="D56" s="12">
+      <c r="D56" s="11">
         <v>-0.40488000000000002</v>
       </c>
-      <c r="E56" s="12">
+      <c r="E56" s="11">
         <v>-1.4094899999999999</v>
       </c>
-      <c r="F56" s="12">
+      <c r="F56" s="11">
         <v>0.10223</v>
       </c>
-      <c r="G56" s="13">
+      <c r="G56" s="12">
         <v>0.94955999999999996</v>
       </c>
-      <c r="H56" s="12">
+      <c r="H56" s="11">
         <v>-1.26915</v>
       </c>
-      <c r="I56" s="12">
+      <c r="I56" s="11">
         <v>-0.27066000000000001</v>
       </c>
-      <c r="J56" s="12">
+      <c r="J56" s="11">
         <v>-0.20035</v>
       </c>
-      <c r="K56" s="12">
+      <c r="K56" s="11">
         <v>1.83901</v>
       </c>
-      <c r="L56" s="12">
+      <c r="L56" s="11">
         <v>-0.41160999999999998</v>
       </c>
-      <c r="M56" s="12">
+      <c r="M56" s="11">
         <v>-0.21590999999999999</v>
       </c>
     </row>
-    <row r="57" spans="1:13">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B57" s="12">
+      <c r="B57" s="11">
         <v>-1.3135699999999999</v>
       </c>
-      <c r="C57" s="12">
+      <c r="C57" s="11">
         <v>0.37391999999999997</v>
       </c>
-      <c r="D57" s="12">
+      <c r="D57" s="11">
         <v>-1.16716</v>
       </c>
-      <c r="E57" s="12">
+      <c r="E57" s="11">
         <v>-1.5136700000000001</v>
       </c>
-      <c r="F57" s="12">
+      <c r="F57" s="11">
         <v>0.26688000000000001</v>
       </c>
-      <c r="G57" s="13">
+      <c r="G57" s="12">
         <v>0.52410999999999996</v>
       </c>
-      <c r="H57" s="12">
+      <c r="H57" s="11">
         <v>-1.7075</v>
       </c>
-      <c r="I57" s="12">
+      <c r="I57" s="11">
         <v>-0.47443000000000002</v>
       </c>
-      <c r="J57" s="12">
+      <c r="J57" s="11">
         <v>-0.47203000000000001</v>
       </c>
-      <c r="K57" s="12">
+      <c r="K57" s="11">
         <v>3.1278000000000001</v>
       </c>
-      <c r="L57" s="12">
+      <c r="L57" s="11">
         <v>-0.22675000000000001</v>
       </c>
-      <c r="M57" s="12">
+      <c r="M57" s="11">
         <v>-0.36975000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:13">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B58" s="12">
+      <c r="B58" s="11">
         <v>-0.53234999999999999</v>
       </c>
-      <c r="C58" s="12">
+      <c r="C58" s="11">
         <v>2.3776700000000002</v>
       </c>
-      <c r="D58" s="12">
+      <c r="D58" s="11">
         <v>7.8219999999999998E-2</v>
       </c>
-      <c r="E58" s="12">
+      <c r="E58" s="11">
         <v>-0.66383000000000003</v>
       </c>
-      <c r="F58" s="12">
+      <c r="F58" s="11">
         <v>0.33683999999999997</v>
       </c>
-      <c r="G58" s="13">
+      <c r="G58" s="12">
         <v>1.2196499999999999</v>
       </c>
-      <c r="H58" s="12">
+      <c r="H58" s="11">
         <v>-0.57540000000000002</v>
       </c>
-      <c r="I58" s="12">
+      <c r="I58" s="11">
         <v>-0.68783000000000005</v>
       </c>
-      <c r="J58" s="12">
+      <c r="J58" s="11">
         <v>0.23995</v>
       </c>
-      <c r="K58" s="12">
+      <c r="K58" s="11">
         <v>2.2132800000000001</v>
       </c>
-      <c r="L58" s="12">
+      <c r="L58" s="11">
         <v>-0.32940999999999998</v>
       </c>
-      <c r="M58" s="12">
+      <c r="M58" s="11">
         <v>-9.2759999999999995E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:13">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B59" s="14">
+      <c r="B59" s="13">
         <v>-1.31149</v>
       </c>
-      <c r="C59" s="14">
+      <c r="C59" s="13">
         <v>0.94621999999999995</v>
       </c>
-      <c r="D59" s="14">
+      <c r="D59" s="13">
         <v>-0.19608</v>
       </c>
-      <c r="E59" s="14">
+      <c r="E59" s="13">
         <v>-0.84196000000000004</v>
       </c>
-      <c r="F59" s="14">
+      <c r="F59" s="13">
         <v>0.58160999999999996</v>
       </c>
-      <c r="G59" s="15">
+      <c r="G59" s="14">
         <v>1.0717000000000001</v>
       </c>
-      <c r="H59" s="14">
+      <c r="H59" s="13">
         <v>-1.7818400000000001</v>
       </c>
-      <c r="I59" s="14">
+      <c r="I59" s="13">
         <v>0.60296000000000005</v>
       </c>
-      <c r="J59" s="14">
+      <c r="J59" s="13">
         <v>-0.74738000000000004</v>
       </c>
-      <c r="K59" s="14">
+      <c r="K59" s="13">
         <v>1.8788100000000001</v>
       </c>
-      <c r="L59" s="14">
+      <c r="L59" s="13">
         <v>-7.7249999999999999E-2</v>
       </c>
-      <c r="M59" s="14">
+      <c r="M59" s="13">
         <v>-0.10011</v>
       </c>
     </row>
-    <row r="60" spans="1:13">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B60" s="14">
+      <c r="B60" s="13">
         <v>-1.46879</v>
       </c>
-      <c r="C60" s="14">
+      <c r="C60" s="13">
         <v>0.20619999999999999</v>
       </c>
-      <c r="D60" s="14">
+      <c r="D60" s="13">
         <v>0.83204999999999996</v>
       </c>
-      <c r="E60" s="14">
+      <c r="E60" s="13">
         <v>-1.43468</v>
       </c>
-      <c r="F60" s="14">
+      <c r="F60" s="13">
         <v>0.63487000000000005</v>
       </c>
-      <c r="G60" s="15">
+      <c r="G60" s="14">
         <v>0.86353999999999997</v>
       </c>
-      <c r="H60" s="14">
+      <c r="H60" s="13">
         <v>-1.1814899999999999</v>
       </c>
-      <c r="I60" s="14">
+      <c r="I60" s="13">
         <v>0.56422000000000005</v>
       </c>
-      <c r="J60" s="14">
+      <c r="J60" s="13">
         <v>-0.44218000000000002</v>
       </c>
-      <c r="K60" s="14">
+      <c r="K60" s="13">
         <v>1.9666699999999999</v>
       </c>
-      <c r="L60" s="14">
+      <c r="L60" s="13">
         <v>-9.196E-2</v>
       </c>
-      <c r="M60" s="14">
+      <c r="M60" s="13">
         <v>-0.1206</v>
       </c>
     </row>
-    <row r="61" spans="1:13">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B61" s="14">
+      <c r="B61" s="13">
         <v>-1.47496</v>
       </c>
-      <c r="C61" s="14">
+      <c r="C61" s="13">
         <v>1.22488</v>
       </c>
-      <c r="D61" s="14">
+      <c r="D61" s="13">
         <v>0.23929</v>
       </c>
-      <c r="E61" s="14">
+      <c r="E61" s="13">
         <v>-1.0818399999999999</v>
       </c>
-      <c r="F61" s="14">
+      <c r="F61" s="13">
         <v>0.60733000000000004</v>
       </c>
-      <c r="G61" s="15">
+      <c r="G61" s="14">
         <v>0.91662999999999994</v>
       </c>
-      <c r="H61" s="14">
+      <c r="H61" s="13">
         <v>-1.3423099999999999</v>
       </c>
-      <c r="I61" s="14">
+      <c r="I61" s="13">
         <v>0.44553999999999999</v>
       </c>
-      <c r="J61" s="14">
+      <c r="J61" s="13">
         <v>-0.52586999999999995</v>
       </c>
-      <c r="K61" s="14">
+      <c r="K61" s="13">
         <v>1.6542300000000001</v>
       </c>
-      <c r="L61" s="14">
+      <c r="L61" s="13">
         <v>-0.25008999999999998</v>
       </c>
-      <c r="M61" s="14">
+      <c r="M61" s="13">
         <v>-0.11491999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:13">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B62" s="14">
+      <c r="B62" s="13">
         <v>-1.7001599999999999</v>
       </c>
-      <c r="C62" s="14">
+      <c r="C62" s="13">
         <v>1.41371</v>
       </c>
-      <c r="D62" s="14">
+      <c r="D62" s="13">
         <v>-0.33731</v>
       </c>
-      <c r="E62" s="14">
+      <c r="E62" s="13">
         <v>-1.0696699999999999</v>
       </c>
-      <c r="F62" s="14">
+      <c r="F62" s="13">
         <v>0.14996000000000001</v>
       </c>
-      <c r="G62" s="15">
+      <c r="G62" s="14">
         <v>0.44447999999999999</v>
       </c>
-      <c r="H62" s="14">
+      <c r="H62" s="13">
         <v>-1.7134100000000001</v>
       </c>
-      <c r="I62" s="14">
+      <c r="I62" s="13">
         <v>0.60153999999999996</v>
       </c>
-      <c r="J62" s="14">
+      <c r="J62" s="13">
         <v>-0.42414000000000002</v>
       </c>
-      <c r="K62" s="14">
+      <c r="K62" s="13">
         <v>1.8240700000000001</v>
       </c>
-      <c r="L62" s="14">
+      <c r="L62" s="13">
         <v>-1.384E-2</v>
       </c>
-      <c r="M62" s="14">
+      <c r="M62" s="13">
         <v>-0.14673</v>
       </c>
     </row>
-    <row r="63" spans="1:13">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B63" s="14">
+      <c r="B63" s="13">
         <v>-1.9470000000000001</v>
       </c>
-      <c r="C63" s="14">
+      <c r="C63" s="13">
         <v>1.0146200000000001</v>
       </c>
-      <c r="D63" s="14">
+      <c r="D63" s="13">
         <v>-0.32612999999999998</v>
       </c>
-      <c r="E63" s="14">
+      <c r="E63" s="13">
         <v>-1.14788</v>
       </c>
-      <c r="F63" s="14">
+      <c r="F63" s="13">
         <v>0.35003000000000001</v>
       </c>
-      <c r="G63" s="15">
+      <c r="G63" s="14">
         <v>-3.0929999999999999E-2</v>
       </c>
-      <c r="H63" s="14">
+      <c r="H63" s="13">
         <v>-1.72651</v>
       </c>
-      <c r="I63" s="14">
+      <c r="I63" s="13">
         <v>0.68239000000000005</v>
       </c>
-      <c r="J63" s="14">
+      <c r="J63" s="13">
         <v>-0.19922000000000001</v>
       </c>
-      <c r="K63" s="14">
+      <c r="K63" s="13">
         <v>1.24976</v>
       </c>
-      <c r="L63" s="14">
+      <c r="L63" s="13">
         <v>-8.6080000000000004E-2</v>
       </c>
-      <c r="M63" s="14">
+      <c r="M63" s="13">
         <v>-0.21015</v>
       </c>
     </row>
-    <row r="64" spans="1:13">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B64" s="14">
+      <c r="B64" s="13">
         <v>-1.8058000000000001</v>
       </c>
-      <c r="C64" s="14">
+      <c r="C64" s="13">
         <v>0.85258</v>
       </c>
-      <c r="D64" s="14">
+      <c r="D64" s="13">
         <v>0.20258000000000001</v>
       </c>
-      <c r="E64" s="14">
+      <c r="E64" s="13">
         <v>-0.89205999999999996</v>
       </c>
-      <c r="F64" s="14">
+      <c r="F64" s="13">
         <v>0.57845999999999997</v>
       </c>
-      <c r="G64" s="15">
+      <c r="G64" s="14">
         <v>0.51160000000000005</v>
       </c>
-      <c r="H64" s="14">
+      <c r="H64" s="13">
         <v>-1.8330599999999999</v>
       </c>
-      <c r="I64" s="14">
+      <c r="I64" s="13">
         <v>0.56654000000000004</v>
       </c>
-      <c r="J64" s="14">
+      <c r="J64" s="13">
         <v>-0.48502000000000001</v>
       </c>
-      <c r="K64" s="14">
+      <c r="K64" s="13">
         <v>1.79833</v>
       </c>
-      <c r="L64" s="14">
+      <c r="L64" s="13">
         <v>-0.16866999999999999</v>
       </c>
-      <c r="M64" s="14">
+      <c r="M64" s="13">
         <v>-0.20585999999999999</v>
       </c>
     </row>
-    <row r="65" spans="1:14">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B65" s="14">
+      <c r="B65" s="13">
         <v>-1.57548</v>
       </c>
-      <c r="C65" s="14">
+      <c r="C65" s="13">
         <v>0.99522999999999995</v>
       </c>
-      <c r="D65" s="14">
+      <c r="D65" s="13">
         <v>0.24099999999999999</v>
       </c>
-      <c r="E65" s="14">
+      <c r="E65" s="13">
         <v>-0.86407999999999996</v>
       </c>
-      <c r="F65" s="14">
+      <c r="F65" s="13">
         <v>0.45516000000000001</v>
       </c>
-      <c r="G65" s="15">
+      <c r="G65" s="14">
         <v>0.59858999999999996</v>
       </c>
-      <c r="H65" s="14">
+      <c r="H65" s="13">
         <v>-1.4654700000000001</v>
       </c>
-      <c r="I65" s="14">
+      <c r="I65" s="13">
         <v>0.53408999999999995</v>
       </c>
-      <c r="J65" s="14">
+      <c r="J65" s="13">
         <v>-0.19642000000000001</v>
       </c>
-      <c r="K65" s="14">
+      <c r="K65" s="13">
         <v>1.76593</v>
       </c>
-      <c r="L65" s="14">
+      <c r="L65" s="13">
         <v>-0.21804000000000001</v>
       </c>
-      <c r="M65" s="14">
+      <c r="M65" s="13">
         <v>-8.0960000000000004E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:14">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B66" s="14">
+      <c r="B66" s="13">
         <v>-1.47156</v>
       </c>
-      <c r="C66" s="14">
+      <c r="C66" s="13">
         <v>0.91598999999999997</v>
       </c>
-      <c r="D66" s="14">
+      <c r="D66" s="13">
         <v>2.7959999999999999E-2</v>
       </c>
-      <c r="E66" s="14">
+      <c r="E66" s="13">
         <v>-1.11768</v>
       </c>
-      <c r="F66" s="14">
+      <c r="F66" s="13">
         <v>0.41188999999999998</v>
       </c>
-      <c r="G66" s="15">
+      <c r="G66" s="14">
         <v>0.77470000000000006</v>
       </c>
-      <c r="H66" s="14">
+      <c r="H66" s="13">
         <v>-1.3954</v>
       </c>
-      <c r="I66" s="14">
+      <c r="I66" s="13">
         <v>0.55069000000000001</v>
       </c>
-      <c r="J66" s="14">
+      <c r="J66" s="13">
         <v>-0.44295000000000001</v>
       </c>
-      <c r="K66" s="14">
+      <c r="K66" s="13">
         <v>1.9323600000000001</v>
       </c>
-      <c r="L66" s="14">
+      <c r="L66" s="13">
         <v>-0.15634999999999999</v>
       </c>
-      <c r="M66" s="14">
+      <c r="M66" s="13">
         <v>-2.4279999999999999E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:14">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B67" s="14">
+      <c r="B67" s="13">
         <v>-1.58558</v>
       </c>
-      <c r="C67" s="14">
+      <c r="C67" s="13">
         <v>1.6873100000000001</v>
       </c>
-      <c r="D67" s="14">
+      <c r="D67" s="13">
         <v>1.0772299999999999</v>
       </c>
-      <c r="E67" s="14">
+      <c r="E67" s="13">
         <v>-0.70340000000000003</v>
       </c>
-      <c r="F67" s="14">
+      <c r="F67" s="13">
         <v>0.40988999999999998</v>
       </c>
-      <c r="G67" s="15">
+      <c r="G67" s="14">
         <v>0.48648000000000002</v>
       </c>
-      <c r="H67" s="14">
+      <c r="H67" s="13">
         <v>-1.4084700000000001</v>
       </c>
-      <c r="I67" s="14">
+      <c r="I67" s="13">
         <v>0.44081999999999999</v>
       </c>
-      <c r="J67" s="14">
+      <c r="J67" s="13">
         <v>-2.1919999999999999E-2</v>
       </c>
-      <c r="K67" s="14">
+      <c r="K67" s="13">
         <v>1.62103</v>
       </c>
-      <c r="L67" s="14">
+      <c r="L67" s="13">
         <v>-0.10857</v>
       </c>
-      <c r="M67" s="14">
+      <c r="M67" s="13">
         <v>-0.13672999999999999</v>
       </c>
     </row>
-    <row r="68" spans="1:14">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B68" s="14">
+      <c r="B68" s="13">
         <v>-1.2528600000000001</v>
       </c>
-      <c r="C68" s="14">
+      <c r="C68" s="13">
         <v>0.93096999999999996</v>
       </c>
-      <c r="D68" s="14">
+      <c r="D68" s="13">
         <v>1.19156</v>
       </c>
-      <c r="E68" s="14">
+      <c r="E68" s="13">
         <v>-0.72248999999999997</v>
       </c>
-      <c r="F68" s="14">
+      <c r="F68" s="13">
         <v>0.68572</v>
       </c>
-      <c r="G68" s="15">
+      <c r="G68" s="14">
         <v>1.12134</v>
       </c>
-      <c r="H68" s="14">
+      <c r="H68" s="13">
         <v>-1.3321499999999999</v>
       </c>
-      <c r="I68" s="14">
+      <c r="I68" s="13">
         <v>0.33384000000000003</v>
       </c>
-      <c r="J68" s="14">
+      <c r="J68" s="13">
         <v>-0.22733999999999999</v>
       </c>
-      <c r="K68" s="14">
+      <c r="K68" s="13">
         <v>1.71817</v>
       </c>
-      <c r="L68" s="14">
+      <c r="L68" s="13">
         <v>-0.1225</v>
       </c>
-      <c r="M68" s="14">
+      <c r="M68" s="13">
         <v>-5.4960000000000002E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:14">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B69" s="14">
+      <c r="B69" s="13">
         <v>-1.85039</v>
       </c>
-      <c r="C69" s="14">
+      <c r="C69" s="13">
         <v>1.02996</v>
       </c>
-      <c r="D69" s="14">
+      <c r="D69" s="13">
         <v>1.2330000000000001E-2</v>
       </c>
-      <c r="E69" s="14">
+      <c r="E69" s="13">
         <v>-0.74944999999999995</v>
       </c>
-      <c r="F69" s="14">
+      <c r="F69" s="13">
         <v>0.20754</v>
       </c>
-      <c r="G69" s="15">
+      <c r="G69" s="14">
         <v>0.24284</v>
       </c>
-      <c r="H69" s="14">
+      <c r="H69" s="13">
         <v>-1.5712299999999999</v>
       </c>
-      <c r="I69" s="14">
+      <c r="I69" s="13">
         <v>0.34949999999999998</v>
       </c>
-      <c r="J69" s="14">
+      <c r="J69" s="13">
         <v>-0.4168</v>
       </c>
-      <c r="K69" s="14">
+      <c r="K69" s="13">
         <v>1.2729699999999999</v>
       </c>
-      <c r="L69" s="14">
+      <c r="L69" s="13">
         <v>-0.18598999999999999</v>
       </c>
-      <c r="M69" s="14">
+      <c r="M69" s="13">
         <v>-0.28965000000000002</v>
       </c>
     </row>
-    <row r="70" spans="1:14">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B70" s="14">
+      <c r="B70" s="13">
         <v>-1.45834</v>
       </c>
-      <c r="C70" s="14">
+      <c r="C70" s="13">
         <v>1.22237</v>
       </c>
-      <c r="D70" s="14">
+      <c r="D70" s="13">
         <v>0.23799000000000001</v>
       </c>
-      <c r="E70" s="14">
+      <c r="E70" s="13">
         <v>-0.83570999999999995</v>
       </c>
-      <c r="F70" s="14">
+      <c r="F70" s="13">
         <v>0.30564999999999998</v>
       </c>
-      <c r="G70" s="15">
+      <c r="G70" s="14">
         <v>0.88924000000000003</v>
       </c>
-      <c r="H70" s="14">
+      <c r="H70" s="13">
         <v>-1.58524</v>
       </c>
-      <c r="I70" s="14">
+      <c r="I70" s="13">
         <v>0.46234999999999998</v>
       </c>
-      <c r="J70" s="14">
+      <c r="J70" s="13">
         <v>-0.56679000000000002</v>
       </c>
-      <c r="K70" s="14">
+      <c r="K70" s="13">
         <v>2.00007</v>
       </c>
-      <c r="L70" s="14">
+      <c r="L70" s="13">
         <v>-7.8020000000000006E-2</v>
       </c>
-      <c r="M70" s="14">
+      <c r="M70" s="13">
         <v>2.818E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:14">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B71" s="14">
+      <c r="B71" s="13">
         <v>-1.19163</v>
       </c>
-      <c r="C71" s="14">
+      <c r="C71" s="13">
         <v>0.92762</v>
       </c>
-      <c r="D71" s="14">
+      <c r="D71" s="13">
         <v>1.0819000000000001</v>
       </c>
-      <c r="E71" s="14">
+      <c r="E71" s="13">
         <v>-1.0128600000000001</v>
       </c>
-      <c r="F71" s="14">
+      <c r="F71" s="13">
         <v>0.72331999999999996</v>
       </c>
-      <c r="G71" s="15">
+      <c r="G71" s="14">
         <v>1.0383</v>
       </c>
-      <c r="H71" s="14">
+      <c r="H71" s="13">
         <v>-1.16934</v>
       </c>
-      <c r="I71" s="14">
+      <c r="I71" s="13">
         <v>0.44219999999999998</v>
       </c>
-      <c r="J71" s="14">
+      <c r="J71" s="13">
         <v>-0.12898999999999999</v>
       </c>
-      <c r="K71" s="14">
+      <c r="K71" s="13">
         <v>1.0847199999999999</v>
       </c>
-      <c r="L71" s="14">
+      <c r="L71" s="13">
         <v>-9.4130000000000005E-2</v>
       </c>
-      <c r="M71" s="14">
+      <c r="M71" s="13">
         <v>-8.9819999999999997E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:14">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B72" s="14">
+      <c r="B72" s="13">
         <v>-1.4866299999999999</v>
       </c>
-      <c r="C72" s="14">
+      <c r="C72" s="13">
         <v>1.30206</v>
       </c>
-      <c r="D72" s="14">
+      <c r="D72" s="13">
         <v>0.12984999999999999</v>
       </c>
-      <c r="E72" s="14">
+      <c r="E72" s="13">
         <v>-1.0191600000000001</v>
       </c>
-      <c r="F72" s="14">
+      <c r="F72" s="13">
         <v>0.36193999999999998</v>
       </c>
-      <c r="G72" s="15">
+      <c r="G72" s="14">
         <v>0.83679999999999999</v>
       </c>
-      <c r="H72" s="14">
+      <c r="H72" s="13">
         <v>-1.65351</v>
       </c>
-      <c r="I72" s="14">
+      <c r="I72" s="13">
         <v>0.40022000000000002</v>
       </c>
-      <c r="J72" s="14">
+      <c r="J72" s="13">
         <v>-0.71755999999999998</v>
       </c>
-      <c r="K72" s="14">
+      <c r="K72" s="13">
         <v>2.2714500000000002</v>
       </c>
-      <c r="L72" s="14">
+      <c r="L72" s="13">
         <v>-0.10839</v>
       </c>
-      <c r="M72" s="14">
+      <c r="M72" s="13">
         <v>4.2300000000000003E-3</v>
       </c>
     </row>
-    <row r="73" spans="1:14">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B73" s="14">
+      <c r="B73" s="13">
         <v>-1.4370700000000001</v>
       </c>
-      <c r="C73" s="14">
+      <c r="C73" s="13">
         <v>2.0295200000000002</v>
       </c>
-      <c r="D73" s="14">
+      <c r="D73" s="13">
         <v>0.64453000000000005</v>
       </c>
-      <c r="E73" s="14">
+      <c r="E73" s="13">
         <v>-0.60016000000000003</v>
       </c>
-      <c r="F73" s="14">
+      <c r="F73" s="13">
         <v>0.59675</v>
       </c>
-      <c r="G73" s="15">
+      <c r="G73" s="14">
         <v>0.69079999999999997</v>
       </c>
-      <c r="H73" s="14">
+      <c r="H73" s="13">
         <v>-1.4129499999999999</v>
       </c>
-      <c r="I73" s="14">
+      <c r="I73" s="13">
         <v>0.21609999999999999</v>
       </c>
-      <c r="J73" s="14">
+      <c r="J73" s="13">
         <v>-0.15584999999999999</v>
       </c>
-      <c r="K73" s="14">
+      <c r="K73" s="13">
         <v>1.07413</v>
       </c>
-      <c r="L73" s="14">
+      <c r="L73" s="13">
         <v>6.0600000000000003E-3</v>
       </c>
-      <c r="M73" s="14">
+      <c r="M73" s="13">
         <v>-7.0250000000000007E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:14">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N74" s="1"/>
     </row>
-    <row r="75" spans="1:14">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N75" s="1"/>
     </row>
-    <row r="76" spans="1:14">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N76" s="1"/>
     </row>
-    <row r="77" spans="1:14">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N77" s="1"/>
     </row>
-    <row r="78" spans="1:14">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N78" s="1"/>
     </row>
   </sheetData>
@@ -3711,672 +3511,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A923D404-E0B1-4623-8A5A-ABD20B1C5FA6}">
-  <dimension ref="A1:C73"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
-  <cols>
-    <col min="1" max="1" width="15" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="16"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="B1" s="5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C14" s="17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C15" s="17"/>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C16" s="17"/>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C17" s="17"/>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C18" s="17"/>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C19" s="17"/>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C20" s="17"/>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C21" s="17"/>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C22" s="17"/>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C23" s="17"/>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C24" s="17"/>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C25" s="17"/>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C26" s="17"/>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C27" s="17"/>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C28" s="17"/>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C29" s="17">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C30" s="17"/>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C31" s="17"/>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C32" s="17"/>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="A33" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C33" s="17"/>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C34" s="17"/>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C35" s="17"/>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C36" s="17"/>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C37" s="17"/>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C38" s="17"/>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C39" s="17"/>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C40" s="17"/>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C41" s="17"/>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C42" s="17"/>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C43" s="17"/>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C44" s="17"/>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C45" s="17"/>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C46" s="17"/>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C47" s="17"/>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="A48" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C48" s="17"/>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C49" s="17"/>
-    </row>
-    <row r="50" spans="1:3">
-      <c r="A50" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C50" s="17"/>
-    </row>
-    <row r="51" spans="1:3">
-      <c r="A51" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C51" s="17"/>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C52" s="17"/>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C53" s="17"/>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="A54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C54" s="17"/>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C55" s="17"/>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="A56" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C56" s="17"/>
-    </row>
-    <row r="57" spans="1:3">
-      <c r="A57" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C57" s="17"/>
-    </row>
-    <row r="58" spans="1:3">
-      <c r="A58" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C58" s="17"/>
-    </row>
-    <row r="59" spans="1:3">
-      <c r="A59" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C59" s="17">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3">
-      <c r="A60" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C60" s="17"/>
-    </row>
-    <row r="61" spans="1:3">
-      <c r="A61" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C61" s="17"/>
-    </row>
-    <row r="62" spans="1:3">
-      <c r="A62" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C62" s="17"/>
-    </row>
-    <row r="63" spans="1:3">
-      <c r="A63" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C63" s="17"/>
-    </row>
-    <row r="64" spans="1:3">
-      <c r="A64" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C64" s="17"/>
-    </row>
-    <row r="65" spans="1:3">
-      <c r="A65" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C65" s="17"/>
-    </row>
-    <row r="66" spans="1:3">
-      <c r="A66" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C66" s="17"/>
-    </row>
-    <row r="67" spans="1:3">
-      <c r="A67" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C67" s="17"/>
-    </row>
-    <row r="68" spans="1:3">
-      <c r="A68" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C68" s="17"/>
-    </row>
-    <row r="69" spans="1:3">
-      <c r="A69" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C69" s="17"/>
-    </row>
-    <row r="70" spans="1:3">
-      <c r="A70" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C70" s="17"/>
-    </row>
-    <row r="71" spans="1:3">
-      <c r="A71" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C71" s="17"/>
-    </row>
-    <row r="72" spans="1:3">
-      <c r="A72" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C72" s="17"/>
-    </row>
-    <row r="73" spans="1:3">
-      <c r="A73" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C73" s="17"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="C14:C28"/>
-    <mergeCell ref="C29:C58"/>
-    <mergeCell ref="C59:C73"/>
-  </mergeCells>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Update all data Excel files
</commit_message>
<xml_diff>
--- a/Early cancer detection/TS Test.xlsx
+++ b/Early cancer detection/TS Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSoft\Pycharm\PythonProject\PythonProject\Archive\01_tri_cancer_screening\Source code for submission\Early cancer detection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BFEC10C-6828-4873-8F29-D44C191C1AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A37FFB22-772D-44EE-BAAE-7499CE50B446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -85,7 +85,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -108,70 +108,33 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -180,15 +143,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -197,21 +154,17 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -490,98 +443,121 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{8F190665-29C1-4D7B-B443-8CBEA912AB74}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;446eed95-321b-4ee0-ab7e-7f3c1ba22191&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N78"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="14" max="14" width="8.88671875" style="4"/>
+    <col min="1" max="13" width="8.88671875" style="5"/>
+    <col min="14" max="14" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:13">
+      <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:13">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="7">
         <v>-1.41622</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="7">
         <v>-1.35989</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="7">
         <v>0.49380000000000002</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="7">
         <v>-1.5841099999999999</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="7">
         <v>0.49720999999999999</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="7">
         <v>0.57604</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2" s="7">
         <v>-0.40747</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="7">
         <v>-1.2265900000000001</v>
       </c>
-      <c r="J2" s="9">
+      <c r="J2" s="7">
         <v>8.1449999999999995E-2</v>
       </c>
-      <c r="K2" s="9">
+      <c r="K2" s="7">
         <v>3.9453100000000001</v>
       </c>
-      <c r="L2" s="9">
+      <c r="L2" s="7">
         <v>-0.29224</v>
       </c>
-      <c r="M2" s="9">
+      <c r="M2" s="7">
         <v>-5.0499999999999998E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:13">
+      <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="7">
@@ -602,7 +578,7 @@
       <c r="G3" s="7">
         <v>0.91549000000000003</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="7">
         <v>-1.4694</v>
       </c>
       <c r="I3" s="7">
@@ -621,8 +597,8 @@
         <v>0.12911</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:13">
+      <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="7">
@@ -643,7 +619,7 @@
       <c r="G4" s="7">
         <v>0.54825999999999997</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="7">
         <v>-1.6550199999999999</v>
       </c>
       <c r="I4" s="7">
@@ -662,8 +638,8 @@
         <v>0.18670999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:13">
+      <c r="A5" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="7">
@@ -684,7 +660,7 @@
       <c r="G5" s="7">
         <v>1.00159</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="7">
         <v>-1.2565500000000001</v>
       </c>
       <c r="I5" s="7">
@@ -703,8 +679,8 @@
         <v>0.28004000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:13">
+      <c r="A6" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="7">
@@ -725,7 +701,7 @@
       <c r="G6" s="7">
         <v>0.81172999999999995</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <v>-1.6113200000000001</v>
       </c>
       <c r="I6" s="7">
@@ -744,8 +720,8 @@
         <v>0.12698000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:13">
+      <c r="A7" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B7" s="7">
@@ -766,7 +742,7 @@
       <c r="G7" s="7">
         <v>0.73860000000000003</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="7">
         <v>-1.53294</v>
       </c>
       <c r="I7" s="7">
@@ -785,8 +761,8 @@
         <v>0.12474</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:13">
+      <c r="A8" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B8" s="7">
@@ -807,7 +783,7 @@
       <c r="G8" s="7">
         <v>1.01393</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="7">
         <v>-1.3601700000000001</v>
       </c>
       <c r="I8" s="7">
@@ -826,8 +802,8 @@
         <v>0.20910999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:13">
+      <c r="A9" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B9" s="7">
@@ -848,7 +824,7 @@
       <c r="G9" s="7">
         <v>0.58652000000000004</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="7">
         <v>-1.6991499999999999</v>
       </c>
       <c r="I9" s="7">
@@ -867,8 +843,8 @@
         <v>5.8090000000000003E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:13">
+      <c r="A10" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B10" s="7">
@@ -889,7 +865,7 @@
       <c r="G10" s="7">
         <v>0.25361</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="7">
         <v>-1.8179700000000001</v>
       </c>
       <c r="I10" s="7">
@@ -908,8 +884,8 @@
         <v>2.913E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:13">
+      <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="7">
@@ -930,7 +906,7 @@
       <c r="G11" s="7">
         <v>0.88263000000000003</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="7">
         <v>-1.5450999999999999</v>
       </c>
       <c r="I11" s="7">
@@ -949,8 +925,8 @@
         <v>0.14810000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:13">
+      <c r="A12" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B12" s="7">
@@ -971,7 +947,7 @@
       <c r="G12" s="7">
         <v>0.80808999999999997</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="7">
         <v>-1.4275800000000001</v>
       </c>
       <c r="I12" s="7">
@@ -990,8 +966,8 @@
         <v>-6.9339999999999999E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:13">
+      <c r="A13" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B13" s="7">
@@ -1012,7 +988,7 @@
       <c r="G13" s="7">
         <v>0.47039999999999998</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="7">
         <v>-1.72149</v>
       </c>
       <c r="I13" s="7">
@@ -1031,2479 +1007,2479 @@
         <v>6.2239999999999997E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="2">
+    <row r="14" spans="1:13" s="2" customFormat="1">
+      <c r="A14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="6">
         <v>-0.92239000000000004</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="6">
         <v>1.3794900000000001</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="6">
         <v>-0.80149999999999999</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="6">
         <v>5.28E-2</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="6">
         <v>0.63182000000000005</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="6">
         <v>0.25452999999999998</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="6">
         <v>-1.8311200000000001</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="6">
         <v>-0.42242000000000002</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="6">
         <v>0.61245000000000005</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="6">
         <v>1.2560800000000001</v>
       </c>
-      <c r="L14" s="2">
+      <c r="L14" s="6">
         <v>-0.51185000000000003</v>
       </c>
-      <c r="M14" s="2">
+      <c r="M14" s="6">
         <v>-0.12891</v>
       </c>
     </row>
-    <row r="15" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="2">
+    <row r="15" spans="1:13" s="2" customFormat="1">
+      <c r="A15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="6">
         <v>2.9369299999999998</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="6">
         <v>1.32355</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="6">
         <v>-1.4099900000000001</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="6">
         <v>-0.65783000000000003</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="6">
         <v>8.1790000000000002E-2</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G15" s="6">
         <v>-8.1989999999999993E-2</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="6">
         <v>-0.56225000000000003</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="6">
         <v>-0.27133000000000002</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="6">
         <v>0.63438000000000005</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="6">
         <v>2.2447300000000001</v>
       </c>
-      <c r="L15" s="2">
+      <c r="L15" s="6">
         <v>-0.27267999999999998</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="6">
         <v>0.36362</v>
       </c>
     </row>
-    <row r="16" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B16" s="2">
+    <row r="16" spans="1:13" s="2" customFormat="1">
+      <c r="A16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="6">
         <v>1.56942</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="6">
         <v>0.70964000000000005</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="6">
         <v>-1.46147</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="6">
         <v>-0.59494999999999998</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="6">
         <v>-0.16158</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G16" s="6">
         <v>-0.28858</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="6">
         <v>-1.0677000000000001</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="6">
         <v>-0.34122000000000002</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="6">
         <v>0.42444999999999999</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="6">
         <v>2.24193</v>
       </c>
-      <c r="L16" s="2">
+      <c r="L16" s="6">
         <v>-0.34732000000000002</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="6">
         <v>0.10390000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="2">
+    <row r="17" spans="1:13" s="2" customFormat="1">
+      <c r="A17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="6">
         <v>-0.88285000000000002</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="6">
         <v>1.42215</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="6">
         <v>-1.4401999999999999</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="6">
         <v>-0.72763999999999995</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="6">
         <v>0.36224000000000001</v>
       </c>
-      <c r="G17" s="2">
+      <c r="G17" s="6">
         <v>0.33376</v>
       </c>
-      <c r="H17" s="3">
+      <c r="H17" s="6">
         <v>-2.0600299999999998</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="6">
         <v>-0.43874000000000002</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="6">
         <v>0.81827000000000005</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="6">
         <v>2.4324699999999999</v>
       </c>
-      <c r="L17" s="2">
+      <c r="L17" s="6">
         <v>-0.47641</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="6">
         <v>-3.4410000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18" s="2">
+    <row r="18" spans="1:13" s="2" customFormat="1">
+      <c r="A18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="6">
         <v>-1.1285400000000001</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="6">
         <v>0.80188999999999999</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="6">
         <v>-0.34087000000000001</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="6">
         <v>-0.45427000000000001</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="6">
         <v>-2.2110000000000001E-2</v>
       </c>
-      <c r="G18" s="2">
+      <c r="G18" s="6">
         <v>0.35472999999999999</v>
       </c>
-      <c r="H18" s="3">
+      <c r="H18" s="6">
         <v>-1.90063</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18" s="6">
         <v>0.17709</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="6">
         <v>0.60316000000000003</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="6">
         <v>1.8084800000000001</v>
       </c>
-      <c r="L18" s="2">
+      <c r="L18" s="6">
         <v>-6.5180000000000002E-2</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="6">
         <v>1.8579999999999999E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B19" s="2">
+    <row r="19" spans="1:13" s="2" customFormat="1">
+      <c r="A19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="6">
         <v>-0.84755000000000003</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="6">
         <v>1.42147</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="6">
         <v>-1.5162500000000001</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="6">
         <v>-0.20774999999999999</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="6">
         <v>6.2920000000000004E-2</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19" s="6">
         <v>-6.7960000000000007E-2</v>
       </c>
-      <c r="H19" s="3">
+      <c r="H19" s="6">
         <v>-1.99244</v>
       </c>
-      <c r="I19" s="2">
+      <c r="I19" s="6">
         <v>-0.31337999999999999</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="6">
         <v>0.52109000000000005</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="6">
         <v>1.2021999999999999</v>
       </c>
-      <c r="L19" s="2">
+      <c r="L19" s="6">
         <v>-0.35224</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="6">
         <v>-4.2799999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B20" s="2">
+    <row r="20" spans="1:13" s="2" customFormat="1">
+      <c r="A20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="6">
         <v>-0.97179000000000004</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="6">
         <v>0.76341999999999999</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="6">
         <v>-5.8380000000000001E-2</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="6">
         <v>-0.87680000000000002</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F20" s="6">
         <v>0.29910999999999999</v>
       </c>
-      <c r="G20" s="2">
+      <c r="G20" s="6">
         <v>0.38096000000000002</v>
       </c>
-      <c r="H20" s="3">
+      <c r="H20" s="6">
         <v>-2.0371800000000002</v>
       </c>
-      <c r="I20" s="2">
+      <c r="I20" s="6">
         <v>-0.30606</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="6">
         <v>0.40128999999999998</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="6">
         <v>1.9677</v>
       </c>
-      <c r="L20" s="2">
+      <c r="L20" s="6">
         <v>-0.57732000000000006</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="6">
         <v>-0.23998</v>
       </c>
     </row>
-    <row r="21" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21" s="2">
+    <row r="21" spans="1:13" s="2" customFormat="1">
+      <c r="A21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="6">
         <v>0.63563000000000003</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="6">
         <v>1.1203099999999999</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="6">
         <v>-1.1225799999999999</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="6">
         <v>-0.68274999999999997</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21" s="6">
         <v>0.44238</v>
       </c>
-      <c r="G21" s="2">
+      <c r="G21" s="6">
         <v>0.40589999999999998</v>
       </c>
-      <c r="H21" s="3">
+      <c r="H21" s="6">
         <v>-1.1087100000000001</v>
       </c>
-      <c r="I21" s="2">
+      <c r="I21" s="6">
         <v>-0.40450999999999998</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="6">
         <v>0.2477</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="6">
         <v>1.4924999999999999</v>
       </c>
-      <c r="L21" s="2">
+      <c r="L21" s="6">
         <v>-0.75743000000000005</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="6">
         <v>-0.2213</v>
       </c>
     </row>
-    <row r="22" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B22" s="2">
+    <row r="22" spans="1:13" s="2" customFormat="1">
+      <c r="A22" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="6">
         <v>-0.73035000000000005</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="6">
         <v>0.82991999999999999</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="6">
         <v>1.6798299999999999</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="6">
         <v>-0.44440000000000002</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="6">
         <v>0.18781</v>
       </c>
-      <c r="G22" s="2">
+      <c r="G22" s="6">
         <v>2.9409999999999999E-2</v>
       </c>
-      <c r="H22" s="3">
+      <c r="H22" s="6">
         <v>-2.1120999999999999</v>
       </c>
-      <c r="I22" s="2">
+      <c r="I22" s="6">
         <v>-0.53285000000000005</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="6">
         <v>0.78910000000000002</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="6">
         <v>1.7154199999999999</v>
       </c>
-      <c r="L22" s="2">
+      <c r="L22" s="6">
         <v>-0.54829000000000006</v>
       </c>
-      <c r="M22" s="2">
+      <c r="M22" s="6">
         <v>-0.32107000000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B23" s="2">
+    <row r="23" spans="1:13" s="2" customFormat="1">
+      <c r="A23" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23" s="6">
         <v>1.2604200000000001</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="6">
         <v>1.12334</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="6">
         <v>1.6914499999999999</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="6">
         <v>-0.58692999999999995</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="6">
         <v>0.28500999999999999</v>
       </c>
-      <c r="G23" s="2">
+      <c r="G23" s="6">
         <v>-0.56835999999999998</v>
       </c>
-      <c r="H23" s="3">
+      <c r="H23" s="6">
         <v>-0.86478999999999995</v>
       </c>
-      <c r="I23" s="2">
+      <c r="I23" s="6">
         <v>-0.73148000000000002</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="6">
         <v>0.78569999999999995</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="6">
         <v>1.4917199999999999</v>
       </c>
-      <c r="L23" s="2">
+      <c r="L23" s="6">
         <v>-0.60851999999999995</v>
       </c>
-      <c r="M23" s="2">
+      <c r="M23" s="6">
         <v>-0.49713000000000002</v>
       </c>
     </row>
-    <row r="24" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="2">
+    <row r="24" spans="1:13" s="2" customFormat="1">
+      <c r="A24" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="6">
         <v>-1.04311</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="6">
         <v>1.0044999999999999</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="6">
         <v>-0.32007999999999998</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="6">
         <v>-1.30419</v>
       </c>
-      <c r="F24" s="2">
+      <c r="F24" s="6">
         <v>-0.19631000000000001</v>
       </c>
-      <c r="G24" s="2">
+      <c r="G24" s="6">
         <v>-0.79010000000000002</v>
       </c>
-      <c r="H24" s="3">
+      <c r="H24" s="6">
         <v>-1.8764799999999999</v>
       </c>
-      <c r="I24" s="2">
+      <c r="I24" s="6">
         <v>-0.91147999999999996</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="6">
         <v>0.48533999999999999</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="6">
         <v>1.66737</v>
       </c>
-      <c r="L24" s="2">
+      <c r="L24" s="6">
         <v>-0.62841999999999998</v>
       </c>
-      <c r="M24" s="2">
+      <c r="M24" s="6">
         <v>-0.43210999999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B25" s="2">
+    <row r="25" spans="1:13" s="2" customFormat="1">
+      <c r="A25" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="6">
         <v>-0.37469000000000002</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C25" s="6">
         <v>0.74528000000000005</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="6">
         <v>3.3976000000000002</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="6">
         <v>-0.34316000000000002</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="6">
         <v>0.37114000000000003</v>
       </c>
-      <c r="G25" s="2">
+      <c r="G25" s="6">
         <v>-0.45446999999999999</v>
       </c>
-      <c r="H25" s="3">
+      <c r="H25" s="6">
         <v>-1.3649100000000001</v>
       </c>
-      <c r="I25" s="2">
+      <c r="I25" s="6">
         <v>-0.52685000000000004</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="6">
         <v>1.02911</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="6">
         <v>1.6331899999999999</v>
       </c>
-      <c r="L25" s="2">
+      <c r="L25" s="6">
         <v>-0.78080000000000005</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="6">
         <v>-0.34375</v>
       </c>
     </row>
-    <row r="26" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B26" s="2">
+    <row r="26" spans="1:13" s="2" customFormat="1">
+      <c r="A26" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="6">
         <v>-1.35538</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C26" s="6">
         <v>0.14702000000000001</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="6">
         <v>-0.79391</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="6">
         <v>-0.93811</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="6">
         <v>-3.9629999999999999E-2</v>
       </c>
-      <c r="G26" s="2">
+      <c r="G26" s="6">
         <v>-0.44957999999999998</v>
       </c>
-      <c r="H26" s="3">
+      <c r="H26" s="6">
         <v>-1.81559</v>
       </c>
-      <c r="I26" s="2">
+      <c r="I26" s="6">
         <v>-0.79108000000000001</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="6">
         <v>0.59975999999999996</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="6">
         <v>1.33467</v>
       </c>
-      <c r="L26" s="2">
+      <c r="L26" s="6">
         <v>-0.75699000000000005</v>
       </c>
-      <c r="M26" s="2">
+      <c r="M26" s="6">
         <v>-0.41450999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B27" s="2">
+    <row r="27" spans="1:13" s="2" customFormat="1">
+      <c r="A27" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="6">
         <v>-1.29589</v>
       </c>
-      <c r="C27" s="2">
+      <c r="C27" s="6">
         <v>1.6867300000000001</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="6">
         <v>1.29802</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="6">
         <v>-0.38113999999999998</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="6">
         <v>0.35631000000000002</v>
       </c>
-      <c r="G27" s="2">
+      <c r="G27" s="6">
         <v>-0.40061000000000002</v>
       </c>
-      <c r="H27" s="3">
+      <c r="H27" s="6">
         <v>-1.78895</v>
       </c>
-      <c r="I27" s="2">
+      <c r="I27" s="6">
         <v>-0.83664000000000005</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="6">
         <v>0.69416999999999995</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="6">
         <v>1.40594</v>
       </c>
-      <c r="L27" s="2">
+      <c r="L27" s="6">
         <v>-0.45207999999999998</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="6">
         <v>-0.41563</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B28" s="2">
+    <row r="28" spans="1:13">
+      <c r="A28" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28" s="6">
         <v>-0.86736000000000002</v>
       </c>
-      <c r="C28" s="2">
+      <c r="C28" s="6">
         <v>2.4040400000000002</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="6">
         <v>0.43731999999999999</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="6">
         <v>0.2266</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="6">
         <v>0.60102999999999995</v>
       </c>
-      <c r="G28" s="2">
+      <c r="G28" s="6">
         <v>0.14507</v>
       </c>
-      <c r="H28" s="3">
+      <c r="H28" s="6">
         <v>-1.56491</v>
       </c>
-      <c r="I28" s="2">
+      <c r="I28" s="6">
         <v>-0.54640999999999995</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="6">
         <v>0.97214</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="6">
         <v>1.35961</v>
       </c>
-      <c r="L28" s="2">
+      <c r="L28" s="6">
         <v>-0.57132000000000005</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="6">
         <v>-0.38588</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B29" s="11">
+    <row r="29" spans="1:13">
+      <c r="A29" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" s="8">
         <v>-1.2083999999999999</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="8">
         <v>1.2352799999999999</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="8">
         <v>-0.71531999999999996</v>
       </c>
-      <c r="E29" s="11">
+      <c r="E29" s="8">
         <v>-1.1348400000000001</v>
       </c>
-      <c r="F29" s="11">
+      <c r="F29" s="8">
         <v>-0.32958999999999999</v>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="8">
         <v>0.87817999999999996</v>
       </c>
-      <c r="H29" s="11">
+      <c r="H29" s="8">
         <v>-1.10131</v>
       </c>
-      <c r="I29" s="11">
+      <c r="I29" s="8">
         <v>-0.18883</v>
       </c>
-      <c r="J29" s="11">
+      <c r="J29" s="8">
         <v>-3.1579999999999997E-2</v>
       </c>
-      <c r="K29" s="11">
+      <c r="K29" s="8">
         <v>2.2745700000000002</v>
       </c>
-      <c r="L29" s="11">
+      <c r="L29" s="8">
         <v>-0.47336</v>
       </c>
-      <c r="M29" s="11">
+      <c r="M29" s="8">
         <v>-0.24510000000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B30" s="11">
+    <row r="30" spans="1:13">
+      <c r="A30" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B30" s="8">
         <v>-1.22922</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="8">
         <v>1.1311800000000001</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="8">
         <v>-1.00522</v>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="8">
         <v>-1.3686199999999999</v>
       </c>
-      <c r="F30" s="11">
+      <c r="F30" s="8">
         <v>1.736E-2</v>
       </c>
-      <c r="G30" s="12">
+      <c r="G30" s="8">
         <v>0.73768</v>
       </c>
-      <c r="H30" s="11">
+      <c r="H30" s="8">
         <v>-1.18655</v>
       </c>
-      <c r="I30" s="11">
+      <c r="I30" s="8">
         <v>-0.27173999999999998</v>
       </c>
-      <c r="J30" s="11">
+      <c r="J30" s="8">
         <v>-0.18110999999999999</v>
       </c>
-      <c r="K30" s="11">
+      <c r="K30" s="8">
         <v>2.5556700000000001</v>
       </c>
-      <c r="L30" s="11">
+      <c r="L30" s="8">
         <v>-0.18981999999999999</v>
       </c>
-      <c r="M30" s="11">
+      <c r="M30" s="8">
         <v>-0.24629999999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B31" s="11">
+    <row r="31" spans="1:13">
+      <c r="A31" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B31" s="8">
         <v>-0.94613000000000003</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="8">
         <v>1.5626899999999999</v>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="8">
         <v>-0.21631</v>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="8">
         <v>-1.1076900000000001</v>
       </c>
-      <c r="F31" s="11">
+      <c r="F31" s="8">
         <v>0.18626999999999999</v>
       </c>
-      <c r="G31" s="12">
+      <c r="G31" s="8">
         <v>0.74480000000000002</v>
       </c>
-      <c r="H31" s="11">
+      <c r="H31" s="8">
         <v>-0.72624</v>
       </c>
-      <c r="I31" s="11">
+      <c r="I31" s="8">
         <v>-0.45101999999999998</v>
       </c>
-      <c r="J31" s="11">
+      <c r="J31" s="8">
         <v>2.3480000000000001E-2</v>
       </c>
-      <c r="K31" s="11">
+      <c r="K31" s="8">
         <v>1.4542900000000001</v>
       </c>
-      <c r="L31" s="11">
+      <c r="L31" s="8">
         <v>-0.30375000000000002</v>
       </c>
-      <c r="M31" s="11">
+      <c r="M31" s="8">
         <v>-0.21811</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B32" s="11">
+    <row r="32" spans="1:13">
+      <c r="A32" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B32" s="8">
         <v>-0.69503999999999999</v>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="8">
         <v>2.0990600000000001</v>
       </c>
-      <c r="D32" s="11">
+      <c r="D32" s="8">
         <v>8.7059999999999998E-2</v>
       </c>
-      <c r="E32" s="11">
+      <c r="E32" s="8">
         <v>-0.59680999999999995</v>
       </c>
-      <c r="F32" s="11">
+      <c r="F32" s="8">
         <v>0.42318</v>
       </c>
-      <c r="G32" s="12">
+      <c r="G32" s="8">
         <v>1.2300500000000001</v>
       </c>
-      <c r="H32" s="11">
+      <c r="H32" s="8">
         <v>-0.70218999999999998</v>
       </c>
-      <c r="I32" s="11">
+      <c r="I32" s="8">
         <v>-0.45713999999999999</v>
       </c>
-      <c r="J32" s="11">
+      <c r="J32" s="8">
         <v>0.30420000000000003</v>
       </c>
-      <c r="K32" s="11">
+      <c r="K32" s="8">
         <v>1.4106300000000001</v>
       </c>
-      <c r="L32" s="11">
+      <c r="L32" s="8">
         <v>-0.37645000000000001</v>
       </c>
-      <c r="M32" s="11">
+      <c r="M32" s="8">
         <v>-0.13922000000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B33" s="11">
+    <row r="33" spans="1:13">
+      <c r="A33" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" s="8">
         <v>-1.3241000000000001</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="8">
         <v>1.9882899999999999</v>
       </c>
-      <c r="D33" s="11">
+      <c r="D33" s="8">
         <v>-0.26128000000000001</v>
       </c>
-      <c r="E33" s="11">
+      <c r="E33" s="8">
         <v>-0.71528999999999998</v>
       </c>
-      <c r="F33" s="11">
+      <c r="F33" s="8">
         <v>0.28905999999999998</v>
       </c>
-      <c r="G33" s="12">
+      <c r="G33" s="8">
         <v>0.75521000000000005</v>
       </c>
-      <c r="H33" s="11">
+      <c r="H33" s="8">
         <v>-1.3332999999999999</v>
       </c>
-      <c r="I33" s="11">
+      <c r="I33" s="8">
         <v>-0.33825</v>
       </c>
-      <c r="J33" s="11">
+      <c r="J33" s="8">
         <v>-8.0210000000000004E-2</v>
       </c>
-      <c r="K33" s="11">
+      <c r="K33" s="8">
         <v>1.72444</v>
       </c>
-      <c r="L33" s="11">
+      <c r="L33" s="8">
         <v>-0.33254</v>
       </c>
-      <c r="M33" s="11">
+      <c r="M33" s="8">
         <v>-0.28497</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B34" s="11">
+    <row r="34" spans="1:13">
+      <c r="A34" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B34" s="8">
         <v>-1.4680599999999999</v>
       </c>
-      <c r="C34" s="11">
+      <c r="C34" s="8">
         <v>1.71753</v>
       </c>
-      <c r="D34" s="11">
+      <c r="D34" s="8">
         <v>-1.09598</v>
       </c>
-      <c r="E34" s="11">
+      <c r="E34" s="8">
         <v>-1.11009</v>
       </c>
-      <c r="F34" s="11">
+      <c r="F34" s="8">
         <v>5.1049999999999998E-2</v>
       </c>
-      <c r="G34" s="12">
+      <c r="G34" s="8">
         <v>0.63202999999999998</v>
       </c>
-      <c r="H34" s="11">
+      <c r="H34" s="8">
         <v>-1.57125</v>
       </c>
-      <c r="I34" s="11">
+      <c r="I34" s="8">
         <v>-0.41792000000000001</v>
       </c>
-      <c r="J34" s="11">
+      <c r="J34" s="8">
         <v>-0.17868999999999999</v>
       </c>
-      <c r="K34" s="11">
+      <c r="K34" s="8">
         <v>2.2224699999999999</v>
       </c>
-      <c r="L34" s="11">
+      <c r="L34" s="8">
         <v>-0.23222000000000001</v>
       </c>
-      <c r="M34" s="11">
+      <c r="M34" s="8">
         <v>-0.30756</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B35" s="11">
+    <row r="35" spans="1:13">
+      <c r="A35" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="8">
         <v>-1.1748499999999999</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="8">
         <v>1.4761299999999999</v>
       </c>
-      <c r="D35" s="11">
+      <c r="D35" s="8">
         <v>-0.47350999999999999</v>
       </c>
-      <c r="E35" s="11">
+      <c r="E35" s="8">
         <v>-1.11046</v>
       </c>
-      <c r="F35" s="11">
+      <c r="F35" s="8">
         <v>0.26125999999999999</v>
       </c>
-      <c r="G35" s="12">
+      <c r="G35" s="8">
         <v>0.58538000000000001</v>
       </c>
-      <c r="H35" s="11">
+      <c r="H35" s="8">
         <v>-1.12276</v>
       </c>
-      <c r="I35" s="11">
+      <c r="I35" s="8">
         <v>-0.27582000000000001</v>
       </c>
-      <c r="J35" s="11">
+      <c r="J35" s="8">
         <v>0.12417</v>
       </c>
-      <c r="K35" s="11">
+      <c r="K35" s="8">
         <v>1.77888</v>
       </c>
-      <c r="L35" s="11">
+      <c r="L35" s="8">
         <v>-0.33561000000000002</v>
       </c>
-      <c r="M35" s="11">
+      <c r="M35" s="8">
         <v>-0.13908999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B36" s="11">
+    <row r="36" spans="1:13">
+      <c r="A36" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" s="8">
         <v>-1.11957</v>
       </c>
-      <c r="C36" s="11">
+      <c r="C36" s="8">
         <v>1.6997599999999999</v>
       </c>
-      <c r="D36" s="11">
+      <c r="D36" s="8">
         <v>-0.40669</v>
       </c>
-      <c r="E36" s="11">
+      <c r="E36" s="8">
         <v>-0.87021999999999999</v>
       </c>
-      <c r="F36" s="11">
+      <c r="F36" s="8">
         <v>0.28193000000000001</v>
       </c>
-      <c r="G36" s="12">
+      <c r="G36" s="8">
         <v>0.60611999999999999</v>
       </c>
-      <c r="H36" s="11">
+      <c r="H36" s="8">
         <v>-1.03685</v>
       </c>
-      <c r="I36" s="11">
+      <c r="I36" s="8">
         <v>-0.30754999999999999</v>
       </c>
-      <c r="J36" s="11">
+      <c r="J36" s="8">
         <v>9.2179999999999998E-2</v>
       </c>
-      <c r="K36" s="11">
+      <c r="K36" s="8">
         <v>1.6114299999999999</v>
       </c>
-      <c r="L36" s="11">
+      <c r="L36" s="8">
         <v>-0.47638000000000003</v>
       </c>
-      <c r="M36" s="11">
+      <c r="M36" s="8">
         <v>-0.20866999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B37" s="11">
+    <row r="37" spans="1:13">
+      <c r="A37" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B37" s="8">
         <v>-1.1451199999999999</v>
       </c>
-      <c r="C37" s="11">
+      <c r="C37" s="8">
         <v>1.50075</v>
       </c>
-      <c r="D37" s="11">
+      <c r="D37" s="8">
         <v>-0.57738</v>
       </c>
-      <c r="E37" s="11">
+      <c r="E37" s="8">
         <v>-1.0672699999999999</v>
       </c>
-      <c r="F37" s="11">
+      <c r="F37" s="8">
         <v>-0.10653</v>
       </c>
-      <c r="G37" s="12">
+      <c r="G37" s="8">
         <v>0.61477999999999999</v>
       </c>
-      <c r="H37" s="11">
+      <c r="H37" s="8">
         <v>-1.33666</v>
       </c>
-      <c r="I37" s="11">
+      <c r="I37" s="8">
         <v>-0.22048999999999999</v>
       </c>
-      <c r="J37" s="11">
+      <c r="J37" s="8">
         <v>0.51119999999999999</v>
       </c>
-      <c r="K37" s="11">
+      <c r="K37" s="8">
         <v>1.2170399999999999</v>
       </c>
-      <c r="L37" s="11">
+      <c r="L37" s="8">
         <v>-0.13880000000000001</v>
       </c>
-      <c r="M37" s="11">
+      <c r="M37" s="8">
         <v>-0.31235000000000002</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B38" s="11">
+    <row r="38" spans="1:13">
+      <c r="A38" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B38" s="8">
         <v>-1.06541</v>
       </c>
-      <c r="C38" s="11">
+      <c r="C38" s="8">
         <v>1.63192</v>
       </c>
-      <c r="D38" s="11">
+      <c r="D38" s="8">
         <v>-0.44180999999999998</v>
       </c>
-      <c r="E38" s="11">
+      <c r="E38" s="8">
         <v>-0.68652000000000002</v>
       </c>
-      <c r="F38" s="11">
+      <c r="F38" s="8">
         <v>0.31536999999999998</v>
       </c>
-      <c r="G38" s="12">
+      <c r="G38" s="8">
         <v>0.90956999999999999</v>
       </c>
-      <c r="H38" s="11">
+      <c r="H38" s="8">
         <v>-1.3687100000000001</v>
       </c>
-      <c r="I38" s="11">
+      <c r="I38" s="8">
         <v>-0.31591999999999998</v>
       </c>
-      <c r="J38" s="11">
+      <c r="J38" s="8">
         <v>0.72940000000000005</v>
       </c>
-      <c r="K38" s="11">
+      <c r="K38" s="8">
         <v>1.35388</v>
       </c>
-      <c r="L38" s="11">
+      <c r="L38" s="8">
         <v>-0.26573000000000002</v>
       </c>
-      <c r="M38" s="11">
+      <c r="M38" s="8">
         <v>-0.19114999999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B39" s="11">
+    <row r="39" spans="1:13">
+      <c r="A39" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B39" s="8">
         <v>-1.0145599999999999</v>
       </c>
-      <c r="C39" s="11">
+      <c r="C39" s="8">
         <v>1.8247100000000001</v>
       </c>
-      <c r="D39" s="11">
+      <c r="D39" s="8">
         <v>-0.34366999999999998</v>
       </c>
-      <c r="E39" s="11">
+      <c r="E39" s="8">
         <v>-0.75348999999999999</v>
       </c>
-      <c r="F39" s="11">
+      <c r="F39" s="8">
         <v>0.29581000000000002</v>
       </c>
-      <c r="G39" s="12">
+      <c r="G39" s="8">
         <v>1.11954</v>
       </c>
-      <c r="H39" s="11">
+      <c r="H39" s="8">
         <v>-1.2730399999999999</v>
       </c>
-      <c r="I39" s="11">
+      <c r="I39" s="8">
         <v>-0.46</v>
       </c>
-      <c r="J39" s="11">
+      <c r="J39" s="8">
         <v>0.14321999999999999</v>
       </c>
-      <c r="K39" s="11">
+      <c r="K39" s="8">
         <v>1.78315</v>
       </c>
-      <c r="L39" s="11">
+      <c r="L39" s="8">
         <v>-0.44283</v>
       </c>
-      <c r="M39" s="11">
+      <c r="M39" s="8">
         <v>-0.26982</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B40" s="11">
+    <row r="40" spans="1:13">
+      <c r="A40" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B40" s="8">
         <v>-0.96314999999999995</v>
       </c>
-      <c r="C40" s="11">
+      <c r="C40" s="8">
         <v>1.48722</v>
       </c>
-      <c r="D40" s="11">
+      <c r="D40" s="8">
         <v>-0.40483000000000002</v>
       </c>
-      <c r="E40" s="11">
+      <c r="E40" s="8">
         <v>-1.0572900000000001</v>
       </c>
-      <c r="F40" s="11">
+      <c r="F40" s="8">
         <v>0.31053999999999998</v>
       </c>
-      <c r="G40" s="12">
+      <c r="G40" s="8">
         <v>0.94404999999999994</v>
       </c>
-      <c r="H40" s="11">
+      <c r="H40" s="8">
         <v>-0.77400000000000002</v>
       </c>
-      <c r="I40" s="11">
+      <c r="I40" s="8">
         <v>-0.19167999999999999</v>
       </c>
-      <c r="J40" s="11">
+      <c r="J40" s="8">
         <v>0.23351</v>
       </c>
-      <c r="K40" s="11">
+      <c r="K40" s="8">
         <v>1.6425700000000001</v>
       </c>
-      <c r="L40" s="11">
+      <c r="L40" s="8">
         <v>-0.53363000000000005</v>
       </c>
-      <c r="M40" s="11">
+      <c r="M40" s="8">
         <v>-0.12716</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B41" s="11">
+    <row r="41" spans="1:13">
+      <c r="A41" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B41" s="8">
         <v>-0.63161</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="8">
         <v>1.86853</v>
       </c>
-      <c r="D41" s="11">
+      <c r="D41" s="8">
         <v>0.19464000000000001</v>
       </c>
-      <c r="E41" s="11">
+      <c r="E41" s="8">
         <v>-0.60221000000000002</v>
       </c>
-      <c r="F41" s="11">
+      <c r="F41" s="8">
         <v>0.45307999999999998</v>
       </c>
-      <c r="G41" s="12">
+      <c r="G41" s="8">
         <v>1.4004700000000001</v>
       </c>
-      <c r="H41" s="11">
+      <c r="H41" s="8">
         <v>-0.97792999999999997</v>
       </c>
-      <c r="I41" s="11">
+      <c r="I41" s="8">
         <v>-0.42316999999999999</v>
       </c>
-      <c r="J41" s="11">
+      <c r="J41" s="8">
         <v>0.51002000000000003</v>
       </c>
-      <c r="K41" s="11">
+      <c r="K41" s="8">
         <v>2.0363799999999999</v>
       </c>
-      <c r="L41" s="11">
+      <c r="L41" s="8">
         <v>-0.48398999999999998</v>
       </c>
-      <c r="M41" s="11">
+      <c r="M41" s="8">
         <v>-0.14248</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B42" s="11">
+    <row r="42" spans="1:13">
+      <c r="A42" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B42" s="8">
         <v>-1.18218</v>
       </c>
-      <c r="C42" s="11">
+      <c r="C42" s="8">
         <v>1.12557</v>
       </c>
-      <c r="D42" s="11">
+      <c r="D42" s="8">
         <v>-0.71718999999999999</v>
       </c>
-      <c r="E42" s="11">
+      <c r="E42" s="8">
         <v>-1.10965</v>
       </c>
-      <c r="F42" s="11">
+      <c r="F42" s="8">
         <v>0.12035999999999999</v>
       </c>
-      <c r="G42" s="12">
+      <c r="G42" s="8">
         <v>0.70986000000000005</v>
       </c>
-      <c r="H42" s="11">
+      <c r="H42" s="8">
         <v>-1.4820599999999999</v>
       </c>
-      <c r="I42" s="11">
+      <c r="I42" s="8">
         <v>0.13533000000000001</v>
       </c>
-      <c r="J42" s="11">
+      <c r="J42" s="8">
         <v>0.27877999999999997</v>
       </c>
-      <c r="K42" s="11">
+      <c r="K42" s="8">
         <v>2.5474299999999999</v>
       </c>
-      <c r="L42" s="11">
+      <c r="L42" s="8">
         <v>-0.31564999999999999</v>
       </c>
-      <c r="M42" s="11">
+      <c r="M42" s="8">
         <v>-0.18806</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B43" s="11">
+    <row r="43" spans="1:13">
+      <c r="A43" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B43" s="8">
         <v>-0.82169999999999999</v>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="8">
         <v>1.7338499999999999</v>
       </c>
-      <c r="D43" s="11">
+      <c r="D43" s="8">
         <v>-0.47008</v>
       </c>
-      <c r="E43" s="11">
+      <c r="E43" s="8">
         <v>-1.0249600000000001</v>
       </c>
-      <c r="F43" s="11">
+      <c r="F43" s="8">
         <v>0.1736</v>
       </c>
-      <c r="G43" s="12">
+      <c r="G43" s="8">
         <v>0.79713999999999996</v>
       </c>
-      <c r="H43" s="11">
+      <c r="H43" s="8">
         <v>-1.2452099999999999</v>
       </c>
-      <c r="I43" s="11">
+      <c r="I43" s="8">
         <v>-0.31494</v>
       </c>
-      <c r="J43" s="11">
+      <c r="J43" s="8">
         <v>0.31359999999999999</v>
       </c>
-      <c r="K43" s="11">
+      <c r="K43" s="8">
         <v>2.2482799999999998</v>
       </c>
-      <c r="L43" s="11">
+      <c r="L43" s="8">
         <v>-0.24886</v>
       </c>
-      <c r="M43" s="11">
+      <c r="M43" s="8">
         <v>-0.22173000000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B44" s="11">
+    <row r="44" spans="1:13">
+      <c r="A44" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B44" s="8">
         <v>-1.06816</v>
       </c>
-      <c r="C44" s="11">
+      <c r="C44" s="8">
         <v>1.59476</v>
       </c>
-      <c r="D44" s="11">
+      <c r="D44" s="8">
         <v>-0.49431999999999998</v>
       </c>
-      <c r="E44" s="11">
+      <c r="E44" s="8">
         <v>-0.75219000000000003</v>
       </c>
-      <c r="F44" s="11">
+      <c r="F44" s="8">
         <v>0.25952999999999998</v>
       </c>
-      <c r="G44" s="12">
+      <c r="G44" s="8">
         <v>0.70992</v>
       </c>
-      <c r="H44" s="11">
+      <c r="H44" s="8">
         <v>-1.4914799999999999</v>
       </c>
-      <c r="I44" s="11">
+      <c r="I44" s="8">
         <v>-0.18281</v>
       </c>
-      <c r="J44" s="11">
+      <c r="J44" s="8">
         <v>-1.8579999999999999E-2</v>
       </c>
-      <c r="K44" s="11">
+      <c r="K44" s="8">
         <v>1.84633</v>
       </c>
-      <c r="L44" s="11">
+      <c r="L44" s="8">
         <v>-0.3831</v>
       </c>
-      <c r="M44" s="11">
+      <c r="M44" s="8">
         <v>-0.35181000000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B45" s="11">
+    <row r="45" spans="1:13">
+      <c r="A45" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B45" s="8">
         <v>-1.1783999999999999</v>
       </c>
-      <c r="C45" s="11">
+      <c r="C45" s="8">
         <v>1.0932200000000001</v>
       </c>
-      <c r="D45" s="11">
+      <c r="D45" s="8">
         <v>-0.48797000000000001</v>
       </c>
-      <c r="E45" s="11">
+      <c r="E45" s="8">
         <v>-1.19163</v>
       </c>
-      <c r="F45" s="11">
+      <c r="F45" s="8">
         <v>0.14280000000000001</v>
       </c>
-      <c r="G45" s="12">
+      <c r="G45" s="8">
         <v>0.97653000000000001</v>
       </c>
-      <c r="H45" s="11">
+      <c r="H45" s="8">
         <v>-1.5720099999999999</v>
       </c>
-      <c r="I45" s="11">
+      <c r="I45" s="8">
         <v>-0.12823000000000001</v>
       </c>
-      <c r="J45" s="11">
+      <c r="J45" s="8">
         <v>5.101E-2</v>
       </c>
-      <c r="K45" s="11">
+      <c r="K45" s="8">
         <v>2.7487400000000002</v>
       </c>
-      <c r="L45" s="11">
+      <c r="L45" s="8">
         <v>-0.27567000000000003</v>
       </c>
-      <c r="M45" s="11">
+      <c r="M45" s="8">
         <v>-0.36004999999999998</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B46" s="11">
+    <row r="46" spans="1:13">
+      <c r="A46" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B46" s="8">
         <v>-1.0864100000000001</v>
       </c>
-      <c r="C46" s="11">
+      <c r="C46" s="8">
         <v>1.53769</v>
       </c>
-      <c r="D46" s="11">
+      <c r="D46" s="8">
         <v>-0.35320000000000001</v>
       </c>
-      <c r="E46" s="11">
+      <c r="E46" s="8">
         <v>-0.75329999999999997</v>
       </c>
-      <c r="F46" s="11">
+      <c r="F46" s="8">
         <v>0.33706999999999998</v>
       </c>
-      <c r="G46" s="12">
+      <c r="G46" s="8">
         <v>0.87129999999999996</v>
       </c>
-      <c r="H46" s="11">
+      <c r="H46" s="8">
         <v>-1.38297</v>
       </c>
-      <c r="I46" s="11">
+      <c r="I46" s="8">
         <v>-0.20097000000000001</v>
       </c>
-      <c r="J46" s="11">
+      <c r="J46" s="8">
         <v>0.36371999999999999</v>
       </c>
-      <c r="K46" s="11">
+      <c r="K46" s="8">
         <v>1.90002</v>
       </c>
-      <c r="L46" s="11">
+      <c r="L46" s="8">
         <v>-0.39494000000000001</v>
       </c>
-      <c r="M46" s="11">
+      <c r="M46" s="8">
         <v>-0.33035999999999999</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B47" s="11">
+    <row r="47" spans="1:13">
+      <c r="A47" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B47" s="8">
         <v>-1.27504</v>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="8">
         <v>1.61056</v>
       </c>
-      <c r="D47" s="11">
+      <c r="D47" s="8">
         <v>-1.1573500000000001</v>
       </c>
-      <c r="E47" s="11">
+      <c r="E47" s="8">
         <v>-1.23837</v>
       </c>
-      <c r="F47" s="11">
+      <c r="F47" s="8">
         <v>0.1532</v>
       </c>
-      <c r="G47" s="12">
+      <c r="G47" s="8">
         <v>0.44252999999999998</v>
       </c>
-      <c r="H47" s="11">
+      <c r="H47" s="8">
         <v>-1.40662</v>
       </c>
-      <c r="I47" s="11">
+      <c r="I47" s="8">
         <v>-0.3669</v>
       </c>
-      <c r="J47" s="11">
+      <c r="J47" s="8">
         <v>0.17224999999999999</v>
       </c>
-      <c r="K47" s="11">
+      <c r="K47" s="8">
         <v>1.98004</v>
       </c>
-      <c r="L47" s="11">
+      <c r="L47" s="8">
         <v>-0.35621999999999998</v>
       </c>
-      <c r="M47" s="11">
+      <c r="M47" s="8">
         <v>-0.40303</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B48" s="11">
+    <row r="48" spans="1:13">
+      <c r="A48" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B48" s="8">
         <v>-1.16204</v>
       </c>
-      <c r="C48" s="11">
+      <c r="C48" s="8">
         <v>1.49169</v>
       </c>
-      <c r="D48" s="11">
+      <c r="D48" s="8">
         <v>-0.55274000000000001</v>
       </c>
-      <c r="E48" s="11">
+      <c r="E48" s="8">
         <v>-0.84509999999999996</v>
       </c>
-      <c r="F48" s="11">
+      <c r="F48" s="8">
         <v>0.23526</v>
       </c>
-      <c r="G48" s="12">
+      <c r="G48" s="8">
         <v>0.71057000000000003</v>
       </c>
-      <c r="H48" s="11">
+      <c r="H48" s="8">
         <v>-1.62808</v>
       </c>
-      <c r="I48" s="11">
+      <c r="I48" s="8">
         <v>-1.788E-2</v>
       </c>
-      <c r="J48" s="11">
+      <c r="J48" s="8">
         <v>0.33331</v>
       </c>
-      <c r="K48" s="11">
+      <c r="K48" s="8">
         <v>2.02685</v>
       </c>
-      <c r="L48" s="11">
+      <c r="L48" s="8">
         <v>-0.39595999999999998</v>
       </c>
-      <c r="M48" s="11">
+      <c r="M48" s="8">
         <v>-0.28720000000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B49" s="11">
+    <row r="49" spans="1:13">
+      <c r="A49" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B49" s="8">
         <v>-1.05474</v>
       </c>
-      <c r="C49" s="11">
+      <c r="C49" s="8">
         <v>1.2202500000000001</v>
       </c>
-      <c r="D49" s="11">
+      <c r="D49" s="8">
         <v>-0.71267999999999998</v>
       </c>
-      <c r="E49" s="11">
+      <c r="E49" s="8">
         <v>-1.1363700000000001</v>
       </c>
-      <c r="F49" s="11">
+      <c r="F49" s="8">
         <v>0.26416000000000001</v>
       </c>
-      <c r="G49" s="12">
+      <c r="G49" s="8">
         <v>0.73926000000000003</v>
       </c>
-      <c r="H49" s="11">
+      <c r="H49" s="8">
         <v>-1.33325</v>
       </c>
-      <c r="I49" s="11">
+      <c r="I49" s="8">
         <v>-0.28577000000000002</v>
       </c>
-      <c r="J49" s="11">
+      <c r="J49" s="8">
         <v>0.24822</v>
       </c>
-      <c r="K49" s="11">
+      <c r="K49" s="8">
         <v>2.4430999999999998</v>
       </c>
-      <c r="L49" s="11">
+      <c r="L49" s="8">
         <v>-0.31785000000000002</v>
       </c>
-      <c r="M49" s="11">
+      <c r="M49" s="8">
         <v>-0.21731</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B50" s="11">
+    <row r="50" spans="1:13">
+      <c r="A50" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50" s="8">
         <v>-0.89812000000000003</v>
       </c>
-      <c r="C50" s="11">
+      <c r="C50" s="8">
         <v>1.5566500000000001</v>
       </c>
-      <c r="D50" s="11">
+      <c r="D50" s="8">
         <v>-0.41810999999999998</v>
       </c>
-      <c r="E50" s="11">
+      <c r="E50" s="8">
         <v>-1.0066600000000001</v>
       </c>
-      <c r="F50" s="11">
+      <c r="F50" s="8">
         <v>0.23608000000000001</v>
       </c>
-      <c r="G50" s="12">
+      <c r="G50" s="8">
         <v>0.98697999999999997</v>
       </c>
-      <c r="H50" s="11">
+      <c r="H50" s="8">
         <v>-1.1273500000000001</v>
       </c>
-      <c r="I50" s="11">
+      <c r="I50" s="8">
         <v>-0.49413000000000001</v>
       </c>
-      <c r="J50" s="11">
+      <c r="J50" s="8">
         <v>9.3700000000000006E-2</v>
       </c>
-      <c r="K50" s="11">
+      <c r="K50" s="8">
         <v>2.1270899999999999</v>
       </c>
-      <c r="L50" s="11">
+      <c r="L50" s="8">
         <v>-0.38144</v>
       </c>
-      <c r="M50" s="11">
+      <c r="M50" s="8">
         <v>-0.35458000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B51" s="11">
+    <row r="51" spans="1:13">
+      <c r="A51" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B51" s="8">
         <v>-1.2175</v>
       </c>
-      <c r="C51" s="11">
+      <c r="C51" s="8">
         <v>2.07335</v>
       </c>
-      <c r="D51" s="11">
+      <c r="D51" s="8">
         <v>-0.12024</v>
       </c>
-      <c r="E51" s="11">
+      <c r="E51" s="8">
         <v>-0.70916999999999997</v>
       </c>
-      <c r="F51" s="11">
+      <c r="F51" s="8">
         <v>0.31714999999999999</v>
       </c>
-      <c r="G51" s="12">
+      <c r="G51" s="8">
         <v>0.69418999999999997</v>
       </c>
-      <c r="H51" s="11">
+      <c r="H51" s="8">
         <v>-0.66805999999999999</v>
       </c>
-      <c r="I51" s="11">
+      <c r="I51" s="8">
         <v>-0.56637999999999999</v>
       </c>
-      <c r="J51" s="11">
+      <c r="J51" s="8">
         <v>0.25722</v>
       </c>
-      <c r="K51" s="11">
+      <c r="K51" s="8">
         <v>0.8861</v>
       </c>
-      <c r="L51" s="11">
+      <c r="L51" s="8">
         <v>-0.66325000000000001</v>
       </c>
-      <c r="M51" s="11">
+      <c r="M51" s="8">
         <v>-0.28621999999999997</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B52" s="11">
+    <row r="52" spans="1:13">
+      <c r="A52" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B52" s="8">
         <v>-0.91959000000000002</v>
       </c>
-      <c r="C52" s="11">
+      <c r="C52" s="8">
         <v>1.34328</v>
       </c>
-      <c r="D52" s="11">
+      <c r="D52" s="8">
         <v>-0.29785</v>
       </c>
-      <c r="E52" s="11">
+      <c r="E52" s="8">
         <v>-0.96106999999999998</v>
       </c>
-      <c r="F52" s="11">
+      <c r="F52" s="8">
         <v>0.38612000000000002</v>
       </c>
-      <c r="G52" s="12">
+      <c r="G52" s="8">
         <v>1.0182800000000001</v>
       </c>
-      <c r="H52" s="11">
+      <c r="H52" s="8">
         <v>-1.23383</v>
       </c>
-      <c r="I52" s="11">
+      <c r="I52" s="8">
         <v>-2.4049999999999998E-2</v>
       </c>
-      <c r="J52" s="11">
+      <c r="J52" s="8">
         <v>0.35155999999999998</v>
       </c>
-      <c r="K52" s="11">
+      <c r="K52" s="8">
         <v>2.3641200000000002</v>
       </c>
-      <c r="L52" s="11">
+      <c r="L52" s="8">
         <v>-0.38159999999999999</v>
       </c>
-      <c r="M52" s="11">
+      <c r="M52" s="8">
         <v>-0.22464000000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B53" s="11">
+    <row r="53" spans="1:13">
+      <c r="A53" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B53" s="8">
         <v>-1.3594999999999999</v>
       </c>
-      <c r="C53" s="11">
+      <c r="C53" s="8">
         <v>1.4438800000000001</v>
       </c>
-      <c r="D53" s="11">
+      <c r="D53" s="8">
         <v>-0.62727999999999995</v>
       </c>
-      <c r="E53" s="11">
+      <c r="E53" s="8">
         <v>-0.91842999999999997</v>
       </c>
-      <c r="F53" s="11">
+      <c r="F53" s="8">
         <v>0.19836000000000001</v>
       </c>
-      <c r="G53" s="12">
+      <c r="G53" s="8">
         <v>0.58357999999999999</v>
       </c>
-      <c r="H53" s="11">
+      <c r="H53" s="8">
         <v>-1.1358200000000001</v>
       </c>
-      <c r="I53" s="11">
+      <c r="I53" s="8">
         <v>-0.16575000000000001</v>
       </c>
-      <c r="J53" s="11">
+      <c r="J53" s="8">
         <v>0.25895000000000001</v>
       </c>
-      <c r="K53" s="11">
+      <c r="K53" s="8">
         <v>1.36541</v>
       </c>
-      <c r="L53" s="11">
+      <c r="L53" s="8">
         <v>-0.40958</v>
       </c>
-      <c r="M53" s="11">
+      <c r="M53" s="8">
         <v>-0.24804000000000001</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B54" s="11">
+    <row r="54" spans="1:13">
+      <c r="A54" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B54" s="8">
         <v>-0.89571999999999996</v>
       </c>
-      <c r="C54" s="11">
+      <c r="C54" s="8">
         <v>1.8649</v>
       </c>
-      <c r="D54" s="11">
+      <c r="D54" s="8">
         <v>-0.24401999999999999</v>
       </c>
-      <c r="E54" s="11">
+      <c r="E54" s="8">
         <v>-0.86006000000000005</v>
       </c>
-      <c r="F54" s="11">
+      <c r="F54" s="8">
         <v>0.42913000000000001</v>
       </c>
-      <c r="G54" s="12">
+      <c r="G54" s="8">
         <v>0.95538999999999996</v>
       </c>
-      <c r="H54" s="11">
+      <c r="H54" s="8">
         <v>-0.97829999999999995</v>
       </c>
-      <c r="I54" s="11">
+      <c r="I54" s="8">
         <v>-0.28028999999999998</v>
       </c>
-      <c r="J54" s="11">
+      <c r="J54" s="8">
         <v>0.26055</v>
       </c>
-      <c r="K54" s="11">
+      <c r="K54" s="8">
         <v>2.0491799999999998</v>
       </c>
-      <c r="L54" s="11">
+      <c r="L54" s="8">
         <v>-0.34964000000000001</v>
       </c>
-      <c r="M54" s="11">
+      <c r="M54" s="8">
         <v>-0.17927999999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B55" s="11">
+    <row r="55" spans="1:13">
+      <c r="A55" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B55" s="8">
         <v>-1.5230399999999999</v>
       </c>
-      <c r="C55" s="11">
+      <c r="C55" s="8">
         <v>1.47163</v>
       </c>
-      <c r="D55" s="11">
+      <c r="D55" s="8">
         <v>-1.2669999999999999</v>
       </c>
-      <c r="E55" s="11">
+      <c r="E55" s="8">
         <v>-1.3667100000000001</v>
       </c>
-      <c r="F55" s="11">
+      <c r="F55" s="8">
         <v>0.11515</v>
       </c>
-      <c r="G55" s="12">
+      <c r="G55" s="8">
         <v>0.27787000000000001</v>
       </c>
-      <c r="H55" s="11">
+      <c r="H55" s="8">
         <v>-1.17997</v>
       </c>
-      <c r="I55" s="11">
+      <c r="I55" s="8">
         <v>-0.45544000000000001</v>
       </c>
-      <c r="J55" s="11">
+      <c r="J55" s="8">
         <v>-0.11458</v>
       </c>
-      <c r="K55" s="11">
+      <c r="K55" s="8">
         <v>1.7778</v>
       </c>
-      <c r="L55" s="11">
+      <c r="L55" s="8">
         <v>-0.26758999999999999</v>
       </c>
-      <c r="M55" s="11">
+      <c r="M55" s="8">
         <v>-0.28763</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B56" s="11">
+    <row r="56" spans="1:13">
+      <c r="A56" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B56" s="8">
         <v>-1.0745899999999999</v>
       </c>
-      <c r="C56" s="11">
+      <c r="C56" s="8">
         <v>1.2802800000000001</v>
       </c>
-      <c r="D56" s="11">
+      <c r="D56" s="8">
         <v>-0.40488000000000002</v>
       </c>
-      <c r="E56" s="11">
+      <c r="E56" s="8">
         <v>-1.4094899999999999</v>
       </c>
-      <c r="F56" s="11">
+      <c r="F56" s="8">
         <v>0.10223</v>
       </c>
-      <c r="G56" s="12">
+      <c r="G56" s="8">
         <v>0.94955999999999996</v>
       </c>
-      <c r="H56" s="11">
+      <c r="H56" s="8">
         <v>-1.26915</v>
       </c>
-      <c r="I56" s="11">
+      <c r="I56" s="8">
         <v>-0.27066000000000001</v>
       </c>
-      <c r="J56" s="11">
+      <c r="J56" s="8">
         <v>-0.20035</v>
       </c>
-      <c r="K56" s="11">
+      <c r="K56" s="8">
         <v>1.83901</v>
       </c>
-      <c r="L56" s="11">
+      <c r="L56" s="8">
         <v>-0.41160999999999998</v>
       </c>
-      <c r="M56" s="11">
+      <c r="M56" s="8">
         <v>-0.21590999999999999</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B57" s="11">
+    <row r="57" spans="1:13">
+      <c r="A57" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B57" s="8">
         <v>-1.3135699999999999</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="8">
         <v>0.37391999999999997</v>
       </c>
-      <c r="D57" s="11">
+      <c r="D57" s="8">
         <v>-1.16716</v>
       </c>
-      <c r="E57" s="11">
+      <c r="E57" s="8">
         <v>-1.5136700000000001</v>
       </c>
-      <c r="F57" s="11">
+      <c r="F57" s="8">
         <v>0.26688000000000001</v>
       </c>
-      <c r="G57" s="12">
+      <c r="G57" s="8">
         <v>0.52410999999999996</v>
       </c>
-      <c r="H57" s="11">
+      <c r="H57" s="8">
         <v>-1.7075</v>
       </c>
-      <c r="I57" s="11">
+      <c r="I57" s="8">
         <v>-0.47443000000000002</v>
       </c>
-      <c r="J57" s="11">
+      <c r="J57" s="8">
         <v>-0.47203000000000001</v>
       </c>
-      <c r="K57" s="11">
+      <c r="K57" s="8">
         <v>3.1278000000000001</v>
       </c>
-      <c r="L57" s="11">
+      <c r="L57" s="8">
         <v>-0.22675000000000001</v>
       </c>
-      <c r="M57" s="11">
+      <c r="M57" s="8">
         <v>-0.36975000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B58" s="11">
+    <row r="58" spans="1:13">
+      <c r="A58" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B58" s="8">
         <v>-0.53234999999999999</v>
       </c>
-      <c r="C58" s="11">
+      <c r="C58" s="8">
         <v>2.3776700000000002</v>
       </c>
-      <c r="D58" s="11">
+      <c r="D58" s="8">
         <v>7.8219999999999998E-2</v>
       </c>
-      <c r="E58" s="11">
+      <c r="E58" s="8">
         <v>-0.66383000000000003</v>
       </c>
-      <c r="F58" s="11">
+      <c r="F58" s="8">
         <v>0.33683999999999997</v>
       </c>
-      <c r="G58" s="12">
+      <c r="G58" s="8">
         <v>1.2196499999999999</v>
       </c>
-      <c r="H58" s="11">
+      <c r="H58" s="8">
         <v>-0.57540000000000002</v>
       </c>
-      <c r="I58" s="11">
+      <c r="I58" s="8">
         <v>-0.68783000000000005</v>
       </c>
-      <c r="J58" s="11">
+      <c r="J58" s="8">
         <v>0.23995</v>
       </c>
-      <c r="K58" s="11">
+      <c r="K58" s="8">
         <v>2.2132800000000001</v>
       </c>
-      <c r="L58" s="11">
+      <c r="L58" s="8">
         <v>-0.32940999999999998</v>
       </c>
-      <c r="M58" s="11">
+      <c r="M58" s="8">
         <v>-9.2759999999999995E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B59" s="13">
+    <row r="59" spans="1:13">
+      <c r="A59" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B59" s="7">
         <v>-1.31149</v>
       </c>
-      <c r="C59" s="13">
+      <c r="C59" s="7">
         <v>0.94621999999999995</v>
       </c>
-      <c r="D59" s="13">
+      <c r="D59" s="7">
         <v>-0.19608</v>
       </c>
-      <c r="E59" s="13">
+      <c r="E59" s="7">
         <v>-0.84196000000000004</v>
       </c>
-      <c r="F59" s="13">
+      <c r="F59" s="7">
         <v>0.58160999999999996</v>
       </c>
-      <c r="G59" s="14">
+      <c r="G59" s="7">
         <v>1.0717000000000001</v>
       </c>
-      <c r="H59" s="13">
+      <c r="H59" s="7">
         <v>-1.7818400000000001</v>
       </c>
-      <c r="I59" s="13">
+      <c r="I59" s="7">
         <v>0.60296000000000005</v>
       </c>
-      <c r="J59" s="13">
+      <c r="J59" s="7">
         <v>-0.74738000000000004</v>
       </c>
-      <c r="K59" s="13">
+      <c r="K59" s="7">
         <v>1.8788100000000001</v>
       </c>
-      <c r="L59" s="13">
+      <c r="L59" s="7">
         <v>-7.7249999999999999E-2</v>
       </c>
-      <c r="M59" s="13">
+      <c r="M59" s="7">
         <v>-0.10011</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B60" s="13">
+    <row r="60" spans="1:13">
+      <c r="A60" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B60" s="7">
         <v>-1.46879</v>
       </c>
-      <c r="C60" s="13">
+      <c r="C60" s="7">
         <v>0.20619999999999999</v>
       </c>
-      <c r="D60" s="13">
+      <c r="D60" s="7">
         <v>0.83204999999999996</v>
       </c>
-      <c r="E60" s="13">
+      <c r="E60" s="7">
         <v>-1.43468</v>
       </c>
-      <c r="F60" s="13">
+      <c r="F60" s="7">
         <v>0.63487000000000005</v>
       </c>
-      <c r="G60" s="14">
+      <c r="G60" s="7">
         <v>0.86353999999999997</v>
       </c>
-      <c r="H60" s="13">
+      <c r="H60" s="7">
         <v>-1.1814899999999999</v>
       </c>
-      <c r="I60" s="13">
+      <c r="I60" s="7">
         <v>0.56422000000000005</v>
       </c>
-      <c r="J60" s="13">
+      <c r="J60" s="7">
         <v>-0.44218000000000002</v>
       </c>
-      <c r="K60" s="13">
+      <c r="K60" s="7">
         <v>1.9666699999999999</v>
       </c>
-      <c r="L60" s="13">
+      <c r="L60" s="7">
         <v>-9.196E-2</v>
       </c>
-      <c r="M60" s="13">
+      <c r="M60" s="7">
         <v>-0.1206</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B61" s="13">
+    <row r="61" spans="1:13">
+      <c r="A61" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B61" s="7">
         <v>-1.47496</v>
       </c>
-      <c r="C61" s="13">
+      <c r="C61" s="7">
         <v>1.22488</v>
       </c>
-      <c r="D61" s="13">
+      <c r="D61" s="7">
         <v>0.23929</v>
       </c>
-      <c r="E61" s="13">
+      <c r="E61" s="7">
         <v>-1.0818399999999999</v>
       </c>
-      <c r="F61" s="13">
+      <c r="F61" s="7">
         <v>0.60733000000000004</v>
       </c>
-      <c r="G61" s="14">
+      <c r="G61" s="7">
         <v>0.91662999999999994</v>
       </c>
-      <c r="H61" s="13">
+      <c r="H61" s="7">
         <v>-1.3423099999999999</v>
       </c>
-      <c r="I61" s="13">
+      <c r="I61" s="7">
         <v>0.44553999999999999</v>
       </c>
-      <c r="J61" s="13">
+      <c r="J61" s="7">
         <v>-0.52586999999999995</v>
       </c>
-      <c r="K61" s="13">
+      <c r="K61" s="7">
         <v>1.6542300000000001</v>
       </c>
-      <c r="L61" s="13">
+      <c r="L61" s="7">
         <v>-0.25008999999999998</v>
       </c>
-      <c r="M61" s="13">
+      <c r="M61" s="7">
         <v>-0.11491999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A62" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B62" s="13">
+    <row r="62" spans="1:13">
+      <c r="A62" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B62" s="7">
         <v>-1.7001599999999999</v>
       </c>
-      <c r="C62" s="13">
+      <c r="C62" s="7">
         <v>1.41371</v>
       </c>
-      <c r="D62" s="13">
+      <c r="D62" s="7">
         <v>-0.33731</v>
       </c>
-      <c r="E62" s="13">
+      <c r="E62" s="7">
         <v>-1.0696699999999999</v>
       </c>
-      <c r="F62" s="13">
+      <c r="F62" s="7">
         <v>0.14996000000000001</v>
       </c>
-      <c r="G62" s="14">
+      <c r="G62" s="7">
         <v>0.44447999999999999</v>
       </c>
-      <c r="H62" s="13">
+      <c r="H62" s="7">
         <v>-1.7134100000000001</v>
       </c>
-      <c r="I62" s="13">
+      <c r="I62" s="7">
         <v>0.60153999999999996</v>
       </c>
-      <c r="J62" s="13">
+      <c r="J62" s="7">
         <v>-0.42414000000000002</v>
       </c>
-      <c r="K62" s="13">
+      <c r="K62" s="7">
         <v>1.8240700000000001</v>
       </c>
-      <c r="L62" s="13">
+      <c r="L62" s="7">
         <v>-1.384E-2</v>
       </c>
-      <c r="M62" s="13">
+      <c r="M62" s="7">
         <v>-0.14673</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A63" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B63" s="13">
+    <row r="63" spans="1:13">
+      <c r="A63" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B63" s="7">
         <v>-1.9470000000000001</v>
       </c>
-      <c r="C63" s="13">
+      <c r="C63" s="7">
         <v>1.0146200000000001</v>
       </c>
-      <c r="D63" s="13">
+      <c r="D63" s="7">
         <v>-0.32612999999999998</v>
       </c>
-      <c r="E63" s="13">
+      <c r="E63" s="7">
         <v>-1.14788</v>
       </c>
-      <c r="F63" s="13">
+      <c r="F63" s="7">
         <v>0.35003000000000001</v>
       </c>
-      <c r="G63" s="14">
+      <c r="G63" s="7">
         <v>-3.0929999999999999E-2</v>
       </c>
-      <c r="H63" s="13">
+      <c r="H63" s="7">
         <v>-1.72651</v>
       </c>
-      <c r="I63" s="13">
+      <c r="I63" s="7">
         <v>0.68239000000000005</v>
       </c>
-      <c r="J63" s="13">
+      <c r="J63" s="7">
         <v>-0.19922000000000001</v>
       </c>
-      <c r="K63" s="13">
+      <c r="K63" s="7">
         <v>1.24976</v>
       </c>
-      <c r="L63" s="13">
+      <c r="L63" s="7">
         <v>-8.6080000000000004E-2</v>
       </c>
-      <c r="M63" s="13">
+      <c r="M63" s="7">
         <v>-0.21015</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B64" s="13">
+    <row r="64" spans="1:13">
+      <c r="A64" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B64" s="7">
         <v>-1.8058000000000001</v>
       </c>
-      <c r="C64" s="13">
+      <c r="C64" s="7">
         <v>0.85258</v>
       </c>
-      <c r="D64" s="13">
+      <c r="D64" s="7">
         <v>0.20258000000000001</v>
       </c>
-      <c r="E64" s="13">
+      <c r="E64" s="7">
         <v>-0.89205999999999996</v>
       </c>
-      <c r="F64" s="13">
+      <c r="F64" s="7">
         <v>0.57845999999999997</v>
       </c>
-      <c r="G64" s="14">
+      <c r="G64" s="7">
         <v>0.51160000000000005</v>
       </c>
-      <c r="H64" s="13">
+      <c r="H64" s="7">
         <v>-1.8330599999999999</v>
       </c>
-      <c r="I64" s="13">
+      <c r="I64" s="7">
         <v>0.56654000000000004</v>
       </c>
-      <c r="J64" s="13">
+      <c r="J64" s="7">
         <v>-0.48502000000000001</v>
       </c>
-      <c r="K64" s="13">
+      <c r="K64" s="7">
         <v>1.79833</v>
       </c>
-      <c r="L64" s="13">
+      <c r="L64" s="7">
         <v>-0.16866999999999999</v>
       </c>
-      <c r="M64" s="13">
+      <c r="M64" s="7">
         <v>-0.20585999999999999</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A65" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B65" s="13">
+    <row r="65" spans="1:14">
+      <c r="A65" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B65" s="7">
         <v>-1.57548</v>
       </c>
-      <c r="C65" s="13">
+      <c r="C65" s="7">
         <v>0.99522999999999995</v>
       </c>
-      <c r="D65" s="13">
+      <c r="D65" s="7">
         <v>0.24099999999999999</v>
       </c>
-      <c r="E65" s="13">
+      <c r="E65" s="7">
         <v>-0.86407999999999996</v>
       </c>
-      <c r="F65" s="13">
+      <c r="F65" s="7">
         <v>0.45516000000000001</v>
       </c>
-      <c r="G65" s="14">
+      <c r="G65" s="7">
         <v>0.59858999999999996</v>
       </c>
-      <c r="H65" s="13">
+      <c r="H65" s="7">
         <v>-1.4654700000000001</v>
       </c>
-      <c r="I65" s="13">
+      <c r="I65" s="7">
         <v>0.53408999999999995</v>
       </c>
-      <c r="J65" s="13">
+      <c r="J65" s="7">
         <v>-0.19642000000000001</v>
       </c>
-      <c r="K65" s="13">
+      <c r="K65" s="7">
         <v>1.76593</v>
       </c>
-      <c r="L65" s="13">
+      <c r="L65" s="7">
         <v>-0.21804000000000001</v>
       </c>
-      <c r="M65" s="13">
+      <c r="M65" s="7">
         <v>-8.0960000000000004E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B66" s="13">
+    <row r="66" spans="1:14">
+      <c r="A66" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B66" s="7">
         <v>-1.47156</v>
       </c>
-      <c r="C66" s="13">
+      <c r="C66" s="7">
         <v>0.91598999999999997</v>
       </c>
-      <c r="D66" s="13">
+      <c r="D66" s="7">
         <v>2.7959999999999999E-2</v>
       </c>
-      <c r="E66" s="13">
+      <c r="E66" s="7">
         <v>-1.11768</v>
       </c>
-      <c r="F66" s="13">
+      <c r="F66" s="7">
         <v>0.41188999999999998</v>
       </c>
-      <c r="G66" s="14">
+      <c r="G66" s="7">
         <v>0.77470000000000006</v>
       </c>
-      <c r="H66" s="13">
+      <c r="H66" s="7">
         <v>-1.3954</v>
       </c>
-      <c r="I66" s="13">
+      <c r="I66" s="7">
         <v>0.55069000000000001</v>
       </c>
-      <c r="J66" s="13">
+      <c r="J66" s="7">
         <v>-0.44295000000000001</v>
       </c>
-      <c r="K66" s="13">
+      <c r="K66" s="7">
         <v>1.9323600000000001</v>
       </c>
-      <c r="L66" s="13">
+      <c r="L66" s="7">
         <v>-0.15634999999999999</v>
       </c>
-      <c r="M66" s="13">
+      <c r="M66" s="7">
         <v>-2.4279999999999999E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A67" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B67" s="13">
+    <row r="67" spans="1:14">
+      <c r="A67" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B67" s="7">
         <v>-1.58558</v>
       </c>
-      <c r="C67" s="13">
+      <c r="C67" s="7">
         <v>1.6873100000000001</v>
       </c>
-      <c r="D67" s="13">
+      <c r="D67" s="7">
         <v>1.0772299999999999</v>
       </c>
-      <c r="E67" s="13">
+      <c r="E67" s="7">
         <v>-0.70340000000000003</v>
       </c>
-      <c r="F67" s="13">
+      <c r="F67" s="7">
         <v>0.40988999999999998</v>
       </c>
-      <c r="G67" s="14">
+      <c r="G67" s="7">
         <v>0.48648000000000002</v>
       </c>
-      <c r="H67" s="13">
+      <c r="H67" s="7">
         <v>-1.4084700000000001</v>
       </c>
-      <c r="I67" s="13">
+      <c r="I67" s="7">
         <v>0.44081999999999999</v>
       </c>
-      <c r="J67" s="13">
+      <c r="J67" s="7">
         <v>-2.1919999999999999E-2</v>
       </c>
-      <c r="K67" s="13">
+      <c r="K67" s="7">
         <v>1.62103</v>
       </c>
-      <c r="L67" s="13">
+      <c r="L67" s="7">
         <v>-0.10857</v>
       </c>
-      <c r="M67" s="13">
+      <c r="M67" s="7">
         <v>-0.13672999999999999</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A68" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B68" s="13">
+    <row r="68" spans="1:14">
+      <c r="A68" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B68" s="7">
         <v>-1.2528600000000001</v>
       </c>
-      <c r="C68" s="13">
+      <c r="C68" s="7">
         <v>0.93096999999999996</v>
       </c>
-      <c r="D68" s="13">
+      <c r="D68" s="7">
         <v>1.19156</v>
       </c>
-      <c r="E68" s="13">
+      <c r="E68" s="7">
         <v>-0.72248999999999997</v>
       </c>
-      <c r="F68" s="13">
+      <c r="F68" s="7">
         <v>0.68572</v>
       </c>
-      <c r="G68" s="14">
+      <c r="G68" s="7">
         <v>1.12134</v>
       </c>
-      <c r="H68" s="13">
+      <c r="H68" s="7">
         <v>-1.3321499999999999</v>
       </c>
-      <c r="I68" s="13">
+      <c r="I68" s="7">
         <v>0.33384000000000003</v>
       </c>
-      <c r="J68" s="13">
+      <c r="J68" s="7">
         <v>-0.22733999999999999</v>
       </c>
-      <c r="K68" s="13">
+      <c r="K68" s="7">
         <v>1.71817</v>
       </c>
-      <c r="L68" s="13">
+      <c r="L68" s="7">
         <v>-0.1225</v>
       </c>
-      <c r="M68" s="13">
+      <c r="M68" s="7">
         <v>-5.4960000000000002E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A69" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B69" s="13">
+    <row r="69" spans="1:14">
+      <c r="A69" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B69" s="7">
         <v>-1.85039</v>
       </c>
-      <c r="C69" s="13">
+      <c r="C69" s="7">
         <v>1.02996</v>
       </c>
-      <c r="D69" s="13">
+      <c r="D69" s="7">
         <v>1.2330000000000001E-2</v>
       </c>
-      <c r="E69" s="13">
+      <c r="E69" s="7">
         <v>-0.74944999999999995</v>
       </c>
-      <c r="F69" s="13">
+      <c r="F69" s="7">
         <v>0.20754</v>
       </c>
-      <c r="G69" s="14">
+      <c r="G69" s="7">
         <v>0.24284</v>
       </c>
-      <c r="H69" s="13">
+      <c r="H69" s="7">
         <v>-1.5712299999999999</v>
       </c>
-      <c r="I69" s="13">
+      <c r="I69" s="7">
         <v>0.34949999999999998</v>
       </c>
-      <c r="J69" s="13">
+      <c r="J69" s="7">
         <v>-0.4168</v>
       </c>
-      <c r="K69" s="13">
+      <c r="K69" s="7">
         <v>1.2729699999999999</v>
       </c>
-      <c r="L69" s="13">
+      <c r="L69" s="7">
         <v>-0.18598999999999999</v>
       </c>
-      <c r="M69" s="13">
+      <c r="M69" s="7">
         <v>-0.28965000000000002</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A70" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B70" s="13">
+    <row r="70" spans="1:14">
+      <c r="A70" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B70" s="7">
         <v>-1.45834</v>
       </c>
-      <c r="C70" s="13">
+      <c r="C70" s="7">
         <v>1.22237</v>
       </c>
-      <c r="D70" s="13">
+      <c r="D70" s="7">
         <v>0.23799000000000001</v>
       </c>
-      <c r="E70" s="13">
+      <c r="E70" s="7">
         <v>-0.83570999999999995</v>
       </c>
-      <c r="F70" s="13">
+      <c r="F70" s="7">
         <v>0.30564999999999998</v>
       </c>
-      <c r="G70" s="14">
+      <c r="G70" s="7">
         <v>0.88924000000000003</v>
       </c>
-      <c r="H70" s="13">
+      <c r="H70" s="7">
         <v>-1.58524</v>
       </c>
-      <c r="I70" s="13">
+      <c r="I70" s="7">
         <v>0.46234999999999998</v>
       </c>
-      <c r="J70" s="13">
+      <c r="J70" s="7">
         <v>-0.56679000000000002</v>
       </c>
-      <c r="K70" s="13">
+      <c r="K70" s="7">
         <v>2.00007</v>
       </c>
-      <c r="L70" s="13">
+      <c r="L70" s="7">
         <v>-7.8020000000000006E-2</v>
       </c>
-      <c r="M70" s="13">
+      <c r="M70" s="7">
         <v>2.818E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A71" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B71" s="13">
+    <row r="71" spans="1:14">
+      <c r="A71" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B71" s="7">
         <v>-1.19163</v>
       </c>
-      <c r="C71" s="13">
+      <c r="C71" s="7">
         <v>0.92762</v>
       </c>
-      <c r="D71" s="13">
+      <c r="D71" s="7">
         <v>1.0819000000000001</v>
       </c>
-      <c r="E71" s="13">
+      <c r="E71" s="7">
         <v>-1.0128600000000001</v>
       </c>
-      <c r="F71" s="13">
+      <c r="F71" s="7">
         <v>0.72331999999999996</v>
       </c>
-      <c r="G71" s="14">
+      <c r="G71" s="7">
         <v>1.0383</v>
       </c>
-      <c r="H71" s="13">
+      <c r="H71" s="7">
         <v>-1.16934</v>
       </c>
-      <c r="I71" s="13">
+      <c r="I71" s="7">
         <v>0.44219999999999998</v>
       </c>
-      <c r="J71" s="13">
+      <c r="J71" s="7">
         <v>-0.12898999999999999</v>
       </c>
-      <c r="K71" s="13">
+      <c r="K71" s="7">
         <v>1.0847199999999999</v>
       </c>
-      <c r="L71" s="13">
+      <c r="L71" s="7">
         <v>-9.4130000000000005E-2</v>
       </c>
-      <c r="M71" s="13">
+      <c r="M71" s="7">
         <v>-8.9819999999999997E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B72" s="13">
+    <row r="72" spans="1:14">
+      <c r="A72" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B72" s="7">
         <v>-1.4866299999999999</v>
       </c>
-      <c r="C72" s="13">
+      <c r="C72" s="7">
         <v>1.30206</v>
       </c>
-      <c r="D72" s="13">
+      <c r="D72" s="7">
         <v>0.12984999999999999</v>
       </c>
-      <c r="E72" s="13">
+      <c r="E72" s="7">
         <v>-1.0191600000000001</v>
       </c>
-      <c r="F72" s="13">
+      <c r="F72" s="7">
         <v>0.36193999999999998</v>
       </c>
-      <c r="G72" s="14">
+      <c r="G72" s="7">
         <v>0.83679999999999999</v>
       </c>
-      <c r="H72" s="13">
+      <c r="H72" s="7">
         <v>-1.65351</v>
       </c>
-      <c r="I72" s="13">
+      <c r="I72" s="7">
         <v>0.40022000000000002</v>
       </c>
-      <c r="J72" s="13">
+      <c r="J72" s="7">
         <v>-0.71755999999999998</v>
       </c>
-      <c r="K72" s="13">
+      <c r="K72" s="7">
         <v>2.2714500000000002</v>
       </c>
-      <c r="L72" s="13">
+      <c r="L72" s="7">
         <v>-0.10839</v>
       </c>
-      <c r="M72" s="13">
+      <c r="M72" s="7">
         <v>4.2300000000000003E-3</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A73" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B73" s="13">
+    <row r="73" spans="1:14">
+      <c r="A73" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B73" s="7">
         <v>-1.4370700000000001</v>
       </c>
-      <c r="C73" s="13">
+      <c r="C73" s="7">
         <v>2.0295200000000002</v>
       </c>
-      <c r="D73" s="13">
+      <c r="D73" s="7">
         <v>0.64453000000000005</v>
       </c>
-      <c r="E73" s="13">
+      <c r="E73" s="7">
         <v>-0.60016000000000003</v>
       </c>
-      <c r="F73" s="13">
+      <c r="F73" s="7">
         <v>0.59675</v>
       </c>
-      <c r="G73" s="14">
+      <c r="G73" s="7">
         <v>0.69079999999999997</v>
       </c>
-      <c r="H73" s="13">
+      <c r="H73" s="7">
         <v>-1.4129499999999999</v>
       </c>
-      <c r="I73" s="13">
+      <c r="I73" s="7">
         <v>0.21609999999999999</v>
       </c>
-      <c r="J73" s="13">
+      <c r="J73" s="7">
         <v>-0.15584999999999999</v>
       </c>
-      <c r="K73" s="13">
+      <c r="K73" s="7">
         <v>1.07413</v>
       </c>
-      <c r="L73" s="13">
+      <c r="L73" s="7">
         <v>6.0600000000000003E-3</v>
       </c>
-      <c r="M73" s="13">
+      <c r="M73" s="7">
         <v>-7.0250000000000007E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14">
       <c r="N74" s="1"/>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14">
       <c r="N75" s="1"/>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14">
       <c r="N76" s="1"/>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14">
       <c r="N77" s="1"/>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14">
       <c r="N78" s="1"/>
     </row>
   </sheetData>

</xml_diff>